<commit_message>
Aplicar formato visual al data.xlsx generado
- convert.py: usa openpyxl directamente para escribir con formato
- Header azul (#106EBE), fuente blanca bold 9pt centrada
- Anchos de columna identicos al archivo de referencia
- Auto-filter habilitado en toda la tabla

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -12,6 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hoja1'!$A$1:$O$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Hoja2'!$A$1:$S$208</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,8 +72,13 @@
       <u val="single"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -85,8 +91,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00106EBE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -103,12 +114,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <right style="medium">
+        <color rgb="00FFFFFF"/>
+      </right>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,6 +140,10 @@
     </xf>
     <xf numFmtId="22" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -7198,99 +7218,120 @@
   </sheetPr>
   <dimension ref="A1:S208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="77" customWidth="1" min="3" max="3"/>
+    <col width="40.57" customWidth="1" min="4" max="4"/>
+    <col width="19.57" customWidth="1" min="5" max="5"/>
+    <col width="15.43" customWidth="1" min="6" max="6"/>
+    <col width="17.71" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15.71" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="9.289999999999999" customWidth="1" min="11" max="11"/>
+    <col width="17.71" customWidth="1" min="12" max="12"/>
+    <col width="47.71" customWidth="1" min="13" max="13"/>
+    <col width="255.71" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="35.43" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="24.71" customWidth="1" min="19" max="19"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Work Item Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Iteration Path</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Estados</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Finish Date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Finish Date Chinalco</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Ticket Chinalco</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Ticket SyC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Tipo Caso</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Tipo Evento</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Tipo Estabilización</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
@@ -7321,13 +7362,13 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="8" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="8" t="n">
         <v>45914.79166666666</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="8" t="n">
         <v>46019.79166666666</v>
       </c>
       <c r="J2" t="inlineStr">
@@ -7398,13 +7439,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="8" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -7475,9 +7516,9 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="G4" s="8" t="n"/>
+      <c r="H4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7542,9 +7583,9 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7609,9 +7650,9 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7676,11 +7717,11 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="8" t="n">
         <v>45391.79166666666</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -7749,13 +7790,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="8" t="n">
         <v>45810.79166666666</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H8" s="8" t="n">
         <v>45873.79166666666</v>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I8" s="8" t="n">
         <v>45937.57847222222</v>
       </c>
       <c r="J8" t="inlineStr">
@@ -7830,13 +7871,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="8" t="n">
         <v>45863.71805555555</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="H9" s="8" t="n">
         <v>45863.71805555555</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="8" t="n">
         <v>45901.26458333333</v>
       </c>
       <c r="J9" t="inlineStr">
@@ -7911,13 +7952,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="8" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H10" s="8" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="8" t="n">
         <v>45530.79166666666</v>
       </c>
       <c r="J10" t="inlineStr">
@@ -7994,13 +8035,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="8" t="n">
         <v>45544.79166666666</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="H11" s="8" t="n">
         <v>45544.79166666666</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J11" t="inlineStr">
@@ -8077,13 +8118,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="8" t="n">
         <v>45933.35277777778</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="8" t="n">
         <v>45937.575</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="8" t="n">
         <v>45959.20069444444</v>
       </c>
       <c r="J12" t="inlineStr">
@@ -8158,13 +8199,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="8" t="n">
         <v>45937.58055555556</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="8" t="n">
         <v>45937.58055555556</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="8" t="n">
         <v>45959.20069444444</v>
       </c>
       <c r="J13" t="inlineStr">
@@ -8239,13 +8280,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="8" t="n">
         <v>45414.79166666666</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="8" t="n">
         <v>45431.79166666666</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="8" t="n">
         <v>45426.79166666666</v>
       </c>
       <c r="J14" t="inlineStr">
@@ -8320,13 +8361,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="8" t="n">
         <v>45414.79166666666</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="H15" s="8" t="n">
         <v>45440.79166666666</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J15" t="inlineStr">
@@ -8401,13 +8442,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H16" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="8" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J16" t="inlineStr">
@@ -8485,11 +8526,11 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="8" t="n">
         <v>46073.42986111111</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
@@ -8558,13 +8599,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="8" t="n">
         <v>45704.79166666666</v>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H18" s="8" t="n">
         <v>45715.79166666666</v>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I18" s="8" t="n">
         <v>45728.79166666666</v>
       </c>
       <c r="J18" t="inlineStr">
@@ -8639,13 +8680,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="8" t="n">
         <v>45771.79166666666</v>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="H19" s="8" t="n">
         <v>45774.79166666666</v>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I19" s="8" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J19" t="inlineStr">
@@ -8720,13 +8761,13 @@
           <t>[Ver. 2.23]</t>
         </is>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="8" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H20" s="8" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I20" s="8" t="n">
         <v>45832.42916666667</v>
       </c>
       <c r="J20" t="inlineStr">
@@ -8801,13 +8842,13 @@
           <t>[Ver 4.0]</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="8" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="H21" s="8" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="I21" s="8" t="n">
         <v>45827.79166666666</v>
       </c>
       <c r="J21" t="inlineStr">
@@ -8882,13 +8923,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G22" s="8" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="8" t="n">
         <v>45354.79166666666</v>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I22" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J22" t="inlineStr">
@@ -8979,13 +9020,13 @@
           <t>[Ver.2.4]</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="8" t="n">
         <v>45337.79166666666</v>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="8" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="I23" s="8" t="n">
         <v>45343.79166666666</v>
       </c>
       <c r="J23" t="inlineStr">
@@ -9056,13 +9097,13 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="8" t="n">
         <v>46019.79166666666</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="8" t="n">
         <v>46022.65347222222</v>
       </c>
-      <c r="I24" s="6" t="n">
+      <c r="I24" s="8" t="n">
         <v>46045.65347222222</v>
       </c>
       <c r="J24" t="inlineStr">
@@ -9135,13 +9176,13 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" s="6" t="n">
+      <c r="G25" s="8" t="n">
         <v>46019.79166666666</v>
       </c>
-      <c r="H25" s="6" t="n">
+      <c r="H25" s="8" t="n">
         <v>46021.79166666666</v>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="I25" s="8" t="n">
         <v>46045.65555555555</v>
       </c>
       <c r="J25" t="inlineStr">
@@ -9218,13 +9259,13 @@
           <t>v2.25.3</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n">
+      <c r="G26" s="8" t="n">
         <v>45988.79166666666</v>
       </c>
-      <c r="H26" s="6" t="n">
+      <c r="H26" s="8" t="n">
         <v>45992.59097222222</v>
       </c>
-      <c r="I26" t="inlineStr"/>
+      <c r="I26" s="8" t="n"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -9285,13 +9326,13 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" s="6" t="n">
+      <c r="G27" s="8" t="n">
         <v>45992.42916666667</v>
       </c>
-      <c r="H27" s="6" t="n">
+      <c r="H27" s="8" t="n">
         <v>45991.79166666666</v>
       </c>
-      <c r="I27" s="6" t="n">
+      <c r="I27" s="8" t="n">
         <v>45995.79166666666</v>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -9362,13 +9403,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="G28" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H28" s="6" t="n">
+      <c r="H28" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I28" s="6" t="n">
+      <c r="I28" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J28" t="inlineStr">
@@ -9445,13 +9486,13 @@
           <t>[Ver. 2.20]</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G29" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H29" s="6" t="n">
+      <c r="H29" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I29" s="6" t="n">
+      <c r="I29" s="8" t="n">
         <v>45665.79166666666</v>
       </c>
       <c r="J29" t="inlineStr">
@@ -9526,13 +9567,13 @@
           <t>[Ver. 1.1]</t>
         </is>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G30" s="8" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="H30" s="6" t="n">
+      <c r="H30" s="8" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="I30" s="8" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J30" t="inlineStr">
@@ -9603,13 +9644,13 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" s="6" t="n">
+      <c r="G31" s="8" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H31" s="6" t="n">
+      <c r="H31" s="8" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="I31" s="6" t="n">
+      <c r="I31" s="8" t="n">
         <v>45550.79166666666</v>
       </c>
       <c r="J31" t="inlineStr">
@@ -9682,13 +9723,13 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" s="6" t="n">
+      <c r="G32" s="8" t="n">
         <v>45427.79166666666</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="8" t="n">
         <v>45439.79166666666</v>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="I32" s="8" t="n">
         <v>45440.79166666666</v>
       </c>
       <c r="J32" t="inlineStr">
@@ -9761,13 +9802,13 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" s="6" t="n">
+      <c r="G33" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H33" s="8" t="n">
         <v>45348.79166666666</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="I33" s="8" t="n">
         <v>45354.79166666666</v>
       </c>
       <c r="J33" t="inlineStr">
@@ -9838,13 +9879,13 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" s="6" t="n">
+      <c r="G34" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H34" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I34" s="6" t="n">
+      <c r="I34" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
       <c r="J34" t="inlineStr">
@@ -9917,13 +9958,13 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" s="6" t="n">
+      <c r="G35" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="H35" s="6" t="n">
+      <c r="H35" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I35" s="6" t="n">
+      <c r="I35" s="8" t="n">
         <v>45383.79166666666</v>
       </c>
       <c r="J35" t="inlineStr">
@@ -9996,13 +10037,13 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" s="6" t="n">
+      <c r="G36" s="8" t="n">
         <v>45396.79166666666</v>
       </c>
-      <c r="H36" s="6" t="n">
+      <c r="H36" s="8" t="n">
         <v>45415.79166666666</v>
       </c>
-      <c r="I36" s="6" t="n">
+      <c r="I36" s="8" t="n">
         <v>45415.79166666666</v>
       </c>
       <c r="J36" t="inlineStr">
@@ -10079,13 +10120,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G37" s="6" t="n">
+      <c r="G37" s="8" t="n">
         <v>45911.30347222222</v>
       </c>
-      <c r="H37" s="6" t="n">
+      <c r="H37" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
-      <c r="I37" s="6" t="n">
+      <c r="I37" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J37" t="inlineStr">
@@ -10156,9 +10197,9 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="G38" s="8" t="n"/>
+      <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10227,13 +10268,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G39" s="8" t="n">
         <v>45930.79166666666</v>
       </c>
-      <c r="H39" s="6" t="n">
+      <c r="H39" s="8" t="n">
         <v>45937.45138888889</v>
       </c>
-      <c r="I39" s="6" t="n">
+      <c r="I39" s="8" t="n">
         <v>45937.57986111111</v>
       </c>
       <c r="J39" t="inlineStr">
@@ -10304,9 +10345,9 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10375,11 +10416,11 @@
           <t>[Ver. 2.27]; [Ver. 2.28]</t>
         </is>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="G41" s="8" t="n">
         <v>45991.79166666666</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10448,13 +10489,13 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" s="6" t="n">
+      <c r="G42" s="8" t="n">
         <v>45931.79166666666</v>
       </c>
-      <c r="H42" s="6" t="n">
+      <c r="H42" s="8" t="n">
         <v>46008.79166666666</v>
       </c>
-      <c r="I42" s="6" t="n">
+      <c r="I42" s="8" t="n">
         <v>46008.79166666666</v>
       </c>
       <c r="J42" t="inlineStr">
@@ -10529,13 +10570,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G43" s="6" t="n">
+      <c r="G43" s="8" t="n">
         <v>45854.72638888889</v>
       </c>
-      <c r="H43" s="6" t="n">
+      <c r="H43" s="8" t="n">
         <v>45854.72638888889</v>
       </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="I43" s="8" t="n"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10608,13 +10649,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G44" s="6" t="n">
+      <c r="G44" s="8" t="n">
         <v>45417.79166666666</v>
       </c>
-      <c r="H44" s="6" t="n">
+      <c r="H44" s="8" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="I44" s="6" t="n">
+      <c r="I44" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J44" t="inlineStr">
@@ -10689,13 +10730,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n">
+      <c r="G45" s="8" t="n">
         <v>45426.79166666666</v>
       </c>
-      <c r="H45" s="6" t="n">
+      <c r="H45" s="8" t="n">
         <v>45476.79166666666</v>
       </c>
-      <c r="I45" s="6" t="n">
+      <c r="I45" s="8" t="n">
         <v>45538.79166666666</v>
       </c>
       <c r="J45" t="inlineStr">
@@ -10770,13 +10811,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G46" s="6" t="n">
+      <c r="G46" s="8" t="n">
         <v>45445.79166666666</v>
       </c>
-      <c r="H46" s="6" t="n">
+      <c r="H46" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I46" s="6" t="n">
+      <c r="I46" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J46" t="inlineStr">
@@ -10851,13 +10892,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G47" s="6" t="n">
+      <c r="G47" s="8" t="n">
         <v>45382.79166666666</v>
       </c>
-      <c r="H47" s="6" t="n">
+      <c r="H47" s="8" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="I47" s="6" t="n">
+      <c r="I47" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J47" t="inlineStr">
@@ -10928,13 +10969,13 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" s="6" t="n">
+      <c r="G48" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
-      <c r="H48" s="6" t="n">
+      <c r="H48" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I48" s="6" t="n">
+      <c r="I48" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J48" t="inlineStr">
@@ -11005,13 +11046,13 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" s="6" t="n">
+      <c r="G49" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
-      <c r="H49" s="6" t="n">
+      <c r="H49" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I49" s="6" t="n">
+      <c r="I49" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J49" t="inlineStr">
@@ -11086,11 +11127,11 @@
           <t>[Ver. 1.3]</t>
         </is>
       </c>
-      <c r="G50" s="6" t="n">
+      <c r="G50" s="8" t="n">
         <v>45446.79166666666</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>Wapsa ES</t>
@@ -11163,13 +11204,13 @@
           <t>[Ver. 1.3]</t>
         </is>
       </c>
-      <c r="G51" s="6" t="n">
+      <c r="G51" s="8" t="n">
         <v>45420.79166666666</v>
       </c>
-      <c r="H51" s="6" t="n">
+      <c r="H51" s="8" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="I51" s="6" t="n">
+      <c r="I51" s="8" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J51" t="inlineStr">
@@ -11244,13 +11285,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G52" s="6" t="n">
+      <c r="G52" s="8" t="n">
         <v>45439.79166666666</v>
       </c>
-      <c r="H52" s="6" t="n">
+      <c r="H52" s="8" t="n">
         <v>45482.79166666666</v>
       </c>
-      <c r="I52" s="6" t="n">
+      <c r="I52" s="8" t="n">
         <v>45489.79166666666</v>
       </c>
       <c r="J52" t="inlineStr">
@@ -11325,13 +11366,13 @@
           <t>[Ver. 1.1]</t>
         </is>
       </c>
-      <c r="G53" s="6" t="n">
+      <c r="G53" s="8" t="n">
         <v>45420.79166666666</v>
       </c>
-      <c r="H53" s="6" t="n">
+      <c r="H53" s="8" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I53" s="6" t="n">
+      <c r="I53" s="8" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J53" t="inlineStr">
@@ -11406,13 +11447,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G54" s="6" t="n">
+      <c r="G54" s="8" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="H54" s="6" t="n">
+      <c r="H54" s="8" t="n">
         <v>45901.79166666666</v>
       </c>
-      <c r="I54" s="6" t="n">
+      <c r="I54" s="8" t="n">
         <v>45937.57847222222</v>
       </c>
       <c r="J54" t="inlineStr">
@@ -11487,13 +11528,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G55" s="6" t="n">
+      <c r="G55" s="8" t="n">
         <v>45874.79166666666</v>
       </c>
-      <c r="H55" s="6" t="n">
+      <c r="H55" s="8" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="I55" s="6" t="n">
+      <c r="I55" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J55" t="inlineStr">
@@ -11568,13 +11609,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G56" s="6" t="n">
+      <c r="G56" s="8" t="n">
         <v>45739.79166666666</v>
       </c>
-      <c r="H56" s="6" t="n">
+      <c r="H56" s="8" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I56" s="6" t="n">
+      <c r="I56" s="8" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J56" t="inlineStr">
@@ -11649,13 +11690,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G57" s="6" t="n">
+      <c r="G57" s="8" t="n">
         <v>45724.79166666666</v>
       </c>
-      <c r="H57" s="6" t="n">
+      <c r="H57" s="8" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="I57" s="6" t="n">
+      <c r="I57" s="8" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J57" t="inlineStr">
@@ -11726,13 +11767,13 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" s="6" t="n">
+      <c r="G58" s="8" t="n">
         <v>46022.79166666666</v>
       </c>
-      <c r="H58" s="6" t="n">
+      <c r="H58" s="8" t="n">
         <v>46052.79166666666</v>
       </c>
-      <c r="I58" s="6" t="n">
+      <c r="I58" s="8" t="n">
         <v>46052.79166666666</v>
       </c>
       <c r="J58" t="inlineStr">
@@ -11803,13 +11844,13 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" s="6" t="n">
+      <c r="G59" s="8" t="n">
         <v>45987.11875</v>
       </c>
-      <c r="H59" s="6" t="n">
+      <c r="H59" s="8" t="n">
         <v>45996.11875</v>
       </c>
-      <c r="I59" s="6" t="n">
+      <c r="I59" s="8" t="n">
         <v>45996.11875</v>
       </c>
       <c r="J59" t="inlineStr">
@@ -11884,13 +11925,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G60" s="6" t="n">
+      <c r="G60" s="8" t="n">
         <v>45762.79166666666</v>
       </c>
-      <c r="H60" s="6" t="n">
+      <c r="H60" s="8" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I60" t="inlineStr"/>
+      <c r="I60" s="8" t="n"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -11963,13 +12004,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G61" s="6" t="n">
+      <c r="G61" s="8" t="n">
         <v>45739.79166666666</v>
       </c>
-      <c r="H61" s="6" t="n">
+      <c r="H61" s="8" t="n">
         <v>45822.79166666666</v>
       </c>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" s="8" t="n"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -12042,13 +12083,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G62" s="6" t="n">
+      <c r="G62" s="8" t="n">
         <v>45713.79166666666</v>
       </c>
-      <c r="H62" s="6" t="n">
+      <c r="H62" s="8" t="n">
         <v>45726.79166666666</v>
       </c>
-      <c r="I62" s="6" t="n">
+      <c r="I62" s="8" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J62" t="inlineStr">
@@ -12119,13 +12160,13 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" s="6" t="n">
+      <c r="G63" s="8" t="n">
         <v>45864.14652777778</v>
       </c>
-      <c r="H63" s="6" t="n">
+      <c r="H63" s="8" t="n">
         <v>45873.79166666666</v>
       </c>
-      <c r="I63" s="6" t="n">
+      <c r="I63" s="8" t="n">
         <v>45873.79166666666</v>
       </c>
       <c r="J63" t="inlineStr">
@@ -12192,13 +12233,13 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" s="6" t="n">
+      <c r="G64" s="8" t="n">
         <v>45886.79166666666</v>
       </c>
-      <c r="H64" s="6" t="n">
+      <c r="H64" s="8" t="n">
         <v>45931.79166666666</v>
       </c>
-      <c r="I64" s="6" t="n">
+      <c r="I64" s="8" t="n">
         <v>45930.79166666666</v>
       </c>
       <c r="J64" t="inlineStr">
@@ -12265,13 +12306,13 @@
           <t>[Ver. 2.24.1]</t>
         </is>
       </c>
-      <c r="G65" s="6" t="n">
+      <c r="G65" s="8" t="n">
         <v>45926.29791666667</v>
       </c>
-      <c r="H65" s="6" t="n">
+      <c r="H65" s="8" t="n">
         <v>45927.79166666666</v>
       </c>
-      <c r="I65" s="6" t="n">
+      <c r="I65" s="8" t="n">
         <v>45959.2</v>
       </c>
       <c r="J65" t="inlineStr">
@@ -12346,13 +12387,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G66" s="6" t="n">
+      <c r="G66" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="H66" s="6" t="n">
+      <c r="H66" s="8" t="n">
         <v>45441.79166666666</v>
       </c>
-      <c r="I66" s="6" t="n">
+      <c r="I66" s="8" t="n">
         <v>45522.79166666666</v>
       </c>
       <c r="J66" t="inlineStr">
@@ -12423,13 +12464,13 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" s="6" t="n">
+      <c r="G67" s="8" t="n">
         <v>45517.79166666666</v>
       </c>
-      <c r="H67" s="6" t="n">
+      <c r="H67" s="8" t="n">
         <v>45517.79166666666</v>
       </c>
-      <c r="I67" s="6" t="n">
+      <c r="I67" s="8" t="n">
         <v>45538.79166666666</v>
       </c>
       <c r="J67" t="inlineStr">
@@ -12502,13 +12543,13 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" s="6" t="n">
+      <c r="G68" s="8" t="n">
         <v>45546.79166666666</v>
       </c>
-      <c r="H68" s="6" t="n">
+      <c r="H68" s="8" t="n">
         <v>45546.79166666666</v>
       </c>
-      <c r="I68" s="6" t="n">
+      <c r="I68" s="8" t="n">
         <v>45574.79166666666</v>
       </c>
       <c r="J68" t="inlineStr">
@@ -12581,13 +12622,13 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" s="6" t="n">
+      <c r="G69" s="8" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="H69" s="6" t="n">
+      <c r="H69" s="8" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="I69" s="6" t="n">
+      <c r="I69" s="8" t="n">
         <v>45540.79166666666</v>
       </c>
       <c r="J69" t="inlineStr">
@@ -12658,13 +12699,13 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" s="6" t="n">
+      <c r="G70" s="8" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="H70" s="6" t="n">
+      <c r="H70" s="8" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="I70" s="6" t="n">
+      <c r="I70" s="8" t="n">
         <v>45558.79166666666</v>
       </c>
       <c r="J70" t="inlineStr">
@@ -12739,13 +12780,13 @@
           <t>[Ver 2.25]; [Ver 4.1]</t>
         </is>
       </c>
-      <c r="G71" s="6" t="n">
+      <c r="G71" s="8" t="n">
         <v>45578.79166666666</v>
       </c>
-      <c r="H71" s="6" t="n">
+      <c r="H71" s="8" t="n">
         <v>45904.26666666667</v>
       </c>
-      <c r="I71" s="6" t="n">
+      <c r="I71" s="8" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J71" t="inlineStr">
@@ -12820,13 +12861,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G72" s="6" t="n">
+      <c r="G72" s="8" t="n">
         <v>45643.79166666666</v>
       </c>
-      <c r="H72" s="6" t="n">
+      <c r="H72" s="8" t="n">
         <v>45904.26111111111</v>
       </c>
-      <c r="I72" s="6" t="n">
+      <c r="I72" s="8" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J72" t="inlineStr">
@@ -12901,13 +12942,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G73" s="6" t="n">
+      <c r="G73" s="8" t="n">
         <v>45915.33055555556</v>
       </c>
-      <c r="H73" s="6" t="n">
+      <c r="H73" s="8" t="n">
         <v>45932.30555555555</v>
       </c>
-      <c r="I73" s="6" t="n">
+      <c r="I73" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J73" t="inlineStr">
@@ -12974,13 +13015,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G74" s="6" t="n">
+      <c r="G74" s="8" t="n">
         <v>45915.33055555556</v>
       </c>
-      <c r="H74" s="6" t="n">
+      <c r="H74" s="8" t="n">
         <v>45932.60069444445</v>
       </c>
-      <c r="I74" s="6" t="n">
+      <c r="I74" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J74" t="inlineStr">
@@ -13051,13 +13092,13 @@
           <t>[Ver. 2.24.1]</t>
         </is>
       </c>
-      <c r="G75" s="6" t="n">
+      <c r="G75" s="8" t="n">
         <v>45924.79166666666</v>
       </c>
-      <c r="H75" s="6" t="n">
+      <c r="H75" s="8" t="n">
         <v>45926.29861111111</v>
       </c>
-      <c r="I75" s="6" t="n">
+      <c r="I75" s="8" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J75" t="inlineStr">
@@ -13132,13 +13173,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G76" s="6" t="n">
+      <c r="G76" s="8" t="n">
         <v>45547.79166666666</v>
       </c>
-      <c r="H76" s="6" t="n">
+      <c r="H76" s="8" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="I76" s="6" t="n">
+      <c r="I76" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J76" t="inlineStr">
@@ -13215,13 +13256,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G77" s="6" t="n">
+      <c r="G77" s="8" t="n">
         <v>45545.79166666666</v>
       </c>
-      <c r="H77" s="6" t="n">
+      <c r="H77" s="8" t="n">
         <v>45545.79166666666</v>
       </c>
-      <c r="I77" s="6" t="n">
+      <c r="I77" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J77" t="inlineStr">
@@ -13299,13 +13340,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G78" s="6" t="n">
+      <c r="G78" s="8" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="H78" s="6" t="n">
+      <c r="H78" s="8" t="n">
         <v>45543.79166666666</v>
       </c>
-      <c r="I78" s="6" t="n">
+      <c r="I78" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J78" t="inlineStr">
@@ -13383,13 +13424,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G79" s="6" t="n">
+      <c r="G79" s="8" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H79" s="6" t="n">
+      <c r="H79" s="8" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="I79" s="6" t="n">
+      <c r="I79" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J79" t="inlineStr">
@@ -13460,13 +13501,13 @@
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" s="6" t="n">
+      <c r="G80" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="H80" s="6" t="n">
+      <c r="H80" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I80" s="6" t="n">
+      <c r="I80" s="8" t="n">
         <v>45575.79166666666</v>
       </c>
       <c r="J80" t="inlineStr">
@@ -13543,13 +13584,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G81" s="6" t="n">
+      <c r="G81" s="8" t="n">
         <v>45559.79166666666</v>
       </c>
-      <c r="H81" s="6" t="n">
+      <c r="H81" s="8" t="n">
         <v>45564.79166666666</v>
       </c>
-      <c r="I81" s="6" t="n">
+      <c r="I81" s="8" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J81" t="inlineStr">
@@ -13620,13 +13661,13 @@
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" s="6" t="n">
+      <c r="G82" s="8" t="n">
         <v>45578.79166666666</v>
       </c>
-      <c r="H82" s="6" t="n">
+      <c r="H82" s="8" t="n">
         <v>45585.79166666666</v>
       </c>
-      <c r="I82" s="6" t="n">
+      <c r="I82" s="8" t="n">
         <v>45585.79166666666</v>
       </c>
       <c r="J82" t="inlineStr">
@@ -13697,13 +13738,13 @@
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" s="6" t="n">
+      <c r="G83" s="8" t="n">
         <v>45870.79166666666</v>
       </c>
-      <c r="H83" s="6" t="n">
+      <c r="H83" s="8" t="n">
         <v>45986.79166666666</v>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" s="8" t="n"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>WAPSA Web</t>
@@ -13768,13 +13809,13 @@
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" s="6" t="n">
+      <c r="G84" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="H84" s="6" t="n">
+      <c r="H84" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I84" s="6" t="n">
+      <c r="I84" s="8" t="n">
         <v>45552.79166666666</v>
       </c>
       <c r="J84" t="inlineStr">
@@ -13845,13 +13886,13 @@
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" s="6" t="n">
+      <c r="G85" s="8" t="n">
         <v>45589.79166666666</v>
       </c>
-      <c r="H85" s="6" t="n">
+      <c r="H85" s="8" t="n">
         <v>45589.79166666666</v>
       </c>
-      <c r="I85" s="6" t="n">
+      <c r="I85" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
       <c r="J85" t="inlineStr">
@@ -13928,13 +13969,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G86" s="6" t="n">
+      <c r="G86" s="8" t="n">
         <v>45592.79166666666</v>
       </c>
-      <c r="H86" s="6" t="n">
+      <c r="H86" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I86" s="6" t="n">
+      <c r="I86" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J86" t="inlineStr">
@@ -14005,13 +14046,13 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" s="6" t="n">
+      <c r="G87" s="8" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H87" s="6" t="n">
+      <c r="H87" s="8" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="I87" s="6" t="n">
+      <c r="I87" s="8" t="n">
         <v>45616.79166666666</v>
       </c>
       <c r="J87" t="inlineStr">
@@ -14084,13 +14125,13 @@
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
-      <c r="G88" s="6" t="n">
+      <c r="G88" s="8" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H88" s="6" t="n">
+      <c r="H88" s="8" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I88" s="6" t="n">
+      <c r="I88" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J88" t="inlineStr">
@@ -14161,13 +14202,13 @@
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" s="6" t="n">
+      <c r="G89" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="H89" s="6" t="n">
+      <c r="H89" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I89" s="6" t="n">
+      <c r="I89" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
       <c r="J89" t="inlineStr">
@@ -14238,13 +14279,13 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" s="6" t="n">
+      <c r="G90" s="8" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H90" s="6" t="n">
+      <c r="H90" s="8" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I90" s="6" t="n">
+      <c r="I90" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J90" t="inlineStr">
@@ -14321,13 +14362,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G91" s="6" t="n">
+      <c r="G91" s="8" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="H91" s="6" t="n">
+      <c r="H91" s="8" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I91" s="6" t="n">
+      <c r="I91" s="8" t="n">
         <v>45662.79166666666</v>
       </c>
       <c r="J91" t="inlineStr">
@@ -14398,13 +14439,13 @@
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
-      <c r="G92" s="6" t="n">
+      <c r="G92" s="8" t="n">
         <v>45608.79166666666</v>
       </c>
-      <c r="H92" s="6" t="n">
+      <c r="H92" s="8" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="I92" s="6" t="n">
+      <c r="I92" s="8" t="n">
         <v>45621.79166666666</v>
       </c>
       <c r="J92" t="inlineStr">
@@ -14481,13 +14522,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G93" s="6" t="n">
+      <c r="G93" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="H93" s="6" t="n">
+      <c r="H93" s="8" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I93" s="6" t="n">
+      <c r="I93" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J93" t="inlineStr">
@@ -14562,13 +14603,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G94" s="6" t="n">
+      <c r="G94" s="8" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="H94" s="6" t="n">
+      <c r="H94" s="8" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="I94" s="6" t="n">
+      <c r="I94" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J94" t="inlineStr">
@@ -14643,13 +14684,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G95" s="6" t="n">
+      <c r="G95" s="8" t="n">
         <v>45627.79166666666</v>
       </c>
-      <c r="H95" s="6" t="n">
+      <c r="H95" s="8" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I95" s="6" t="n">
+      <c r="I95" s="8" t="n">
         <v>45671.79166666666</v>
       </c>
       <c r="J95" t="inlineStr">
@@ -14724,13 +14765,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G96" s="6" t="n">
+      <c r="G96" s="8" t="n">
         <v>45623.79166666666</v>
       </c>
-      <c r="H96" s="6" t="n">
+      <c r="H96" s="8" t="n">
         <v>45623.79166666666</v>
       </c>
-      <c r="I96" s="6" t="n">
+      <c r="I96" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J96" t="inlineStr">
@@ -14801,13 +14842,13 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" s="6" t="n">
+      <c r="G97" s="8" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="H97" s="6" t="n">
+      <c r="H97" s="8" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I97" s="6" t="n">
+      <c r="I97" s="8" t="n">
         <v>45680.79166666666</v>
       </c>
       <c r="J97" t="inlineStr">
@@ -14884,13 +14925,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G98" s="6" t="n">
+      <c r="G98" s="8" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="H98" s="6" t="n">
+      <c r="H98" s="8" t="n">
         <v>45389.79166666666</v>
       </c>
-      <c r="I98" s="6" t="n">
+      <c r="I98" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J98" t="inlineStr">
@@ -14961,13 +15002,13 @@
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" s="6" t="n">
+      <c r="G99" s="8" t="n">
         <v>45396.79166666666</v>
       </c>
-      <c r="H99" s="6" t="n">
+      <c r="H99" s="8" t="n">
         <v>45435.79166666666</v>
       </c>
-      <c r="I99" s="6" t="n">
+      <c r="I99" s="8" t="n">
         <v>45435.79166666666</v>
       </c>
       <c r="J99" t="inlineStr">
@@ -15044,13 +15085,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G100" s="6" t="n">
+      <c r="G100" s="8" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="H100" s="6" t="n">
+      <c r="H100" s="8" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="I100" s="6" t="n">
+      <c r="I100" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J100" t="inlineStr">
@@ -15125,13 +15166,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G101" s="6" t="n">
+      <c r="G101" s="8" t="n">
         <v>45398.79166666666</v>
       </c>
-      <c r="H101" s="6" t="n">
+      <c r="H101" s="8" t="n">
         <v>45398.79166666666</v>
       </c>
-      <c r="I101" s="6" t="n">
+      <c r="I101" s="8" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J101" t="inlineStr">
@@ -15206,13 +15247,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G102" s="6" t="n">
+      <c r="G102" s="8" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="H102" s="6" t="n">
+      <c r="H102" s="8" t="n">
         <v>45425.79166666666</v>
       </c>
-      <c r="I102" s="6" t="n">
+      <c r="I102" s="8" t="n">
         <v>45427.79166666666</v>
       </c>
       <c r="J102" t="inlineStr">
@@ -15283,13 +15324,13 @@
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
-      <c r="G103" s="6" t="n">
+      <c r="G103" s="8" t="n">
         <v>45405.79166666666</v>
       </c>
-      <c r="H103" s="6" t="n">
+      <c r="H103" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I103" s="6" t="n">
+      <c r="I103" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
       <c r="J103" t="inlineStr">
@@ -15360,13 +15401,13 @@
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
-      <c r="G104" s="6" t="n">
+      <c r="G104" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="H104" s="6" t="n">
+      <c r="H104" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I104" s="6" t="n">
+      <c r="I104" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
       <c r="J104" t="inlineStr">
@@ -15441,13 +15482,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G105" s="6" t="n">
+      <c r="G105" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="H105" s="6" t="n">
+      <c r="H105" s="8" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I105" s="6" t="n">
+      <c r="I105" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J105" t="inlineStr">
@@ -15522,13 +15563,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G106" s="6" t="n">
+      <c r="G106" s="8" t="n">
         <v>45433.79166666666</v>
       </c>
-      <c r="H106" s="6" t="n">
+      <c r="H106" s="8" t="n">
         <v>45433.79166666666</v>
       </c>
-      <c r="I106" s="6" t="n">
+      <c r="I106" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J106" t="inlineStr">
@@ -15599,13 +15640,13 @@
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
-      <c r="G107" s="6" t="n">
+      <c r="G107" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="H107" s="6" t="n">
+      <c r="H107" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="I107" s="6" t="n">
+      <c r="I107" s="8" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J107" t="inlineStr">
@@ -15680,13 +15721,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G108" s="6" t="n">
+      <c r="G108" s="8" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="H108" s="6" t="n">
+      <c r="H108" s="8" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="I108" s="6" t="n">
+      <c r="I108" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
       <c r="J108" t="inlineStr">
@@ -15763,13 +15804,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G109" s="6" t="n">
+      <c r="G109" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H109" s="6" t="n">
+      <c r="H109" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="I109" s="6" t="n">
+      <c r="I109" s="8" t="n">
         <v>45431.79166666666</v>
       </c>
       <c r="J109" t="inlineStr">
@@ -15844,13 +15885,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G110" s="6" t="n">
+      <c r="G110" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H110" s="6" t="n">
+      <c r="H110" s="8" t="n">
         <v>45361.79166666666</v>
       </c>
-      <c r="I110" s="6" t="n">
+      <c r="I110" s="8" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J110" t="inlineStr">
@@ -15923,13 +15964,13 @@
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
-      <c r="G111" s="6" t="n">
+      <c r="G111" s="8" t="n">
         <v>45368.79166666666</v>
       </c>
-      <c r="H111" s="6" t="n">
+      <c r="H111" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I111" s="6" t="n">
+      <c r="I111" s="8" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J111" t="inlineStr">
@@ -16002,13 +16043,13 @@
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
-      <c r="G112" s="6" t="n">
+      <c r="G112" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="H112" s="6" t="n">
+      <c r="H112" s="8" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I112" s="6" t="n">
+      <c r="I112" s="8" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J112" t="inlineStr">
@@ -16079,11 +16120,11 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" s="6" t="n">
+      <c r="G113" s="8" t="n">
         <v>45951.79166666666</v>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
+      <c r="H113" s="8" t="n"/>
+      <c r="I113" s="8" t="n"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16148,13 +16189,13 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
-      <c r="G114" s="6" t="n">
+      <c r="G114" s="8" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="H114" s="6" t="n">
+      <c r="H114" s="8" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="I114" t="inlineStr"/>
+      <c r="I114" s="8" t="n"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16227,13 +16268,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G115" s="6" t="n">
+      <c r="G115" s="8" t="n">
         <v>45845.25347222222</v>
       </c>
-      <c r="H115" s="6" t="n">
+      <c r="H115" s="8" t="n">
         <v>45845.79166666666</v>
       </c>
-      <c r="I115" t="inlineStr"/>
+      <c r="I115" s="8" t="n"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16310,13 +16351,13 @@
           <t>[Ver. 4.29]</t>
         </is>
       </c>
-      <c r="G116" s="6" t="n">
+      <c r="G116" s="8" t="n">
         <v>46047.79166666666</v>
       </c>
-      <c r="H116" s="6" t="n">
+      <c r="H116" s="8" t="n">
         <v>46104.26111111111</v>
       </c>
-      <c r="I116" t="inlineStr"/>
+      <c r="I116" s="8" t="n"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16385,13 +16426,13 @@
           <t>[Ver. 2.29]</t>
         </is>
       </c>
-      <c r="G117" s="6" t="n">
+      <c r="G117" s="8" t="n">
         <v>46050.79166666666</v>
       </c>
-      <c r="H117" s="6" t="n">
+      <c r="H117" s="8" t="n">
         <v>46062.46458333333</v>
       </c>
-      <c r="I117" t="inlineStr"/>
+      <c r="I117" s="8" t="n"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16460,13 +16501,13 @@
           <t>[Ver. 2.28]; SLA</t>
         </is>
       </c>
-      <c r="G118" s="6" t="n">
+      <c r="G118" s="8" t="n">
         <v>46090.20833333334</v>
       </c>
-      <c r="H118" s="6" t="n">
+      <c r="H118" s="8" t="n">
         <v>46090.33333333334</v>
       </c>
-      <c r="I118" t="inlineStr"/>
+      <c r="I118" s="8" t="n"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16543,11 +16584,11 @@
           <t>[Ver. 2.28]; SLA</t>
         </is>
       </c>
-      <c r="G119" s="6" t="n">
+      <c r="G119" s="8" t="n">
         <v>46089.79166666666</v>
       </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
+      <c r="H119" s="8" t="n"/>
+      <c r="I119" s="8" t="n"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>WapsaWeb</t>
@@ -16612,13 +16653,13 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
-      <c r="G120" s="6" t="n">
+      <c r="G120" s="8" t="n">
         <v>46094.54930555556</v>
       </c>
-      <c r="H120" s="6" t="n">
+      <c r="H120" s="8" t="n">
         <v>46094.54930555556</v>
       </c>
-      <c r="I120" s="6" t="n">
+      <c r="I120" s="8" t="n">
         <v>46097.30972222222</v>
       </c>
       <c r="J120" t="inlineStr">
@@ -16693,13 +16734,13 @@
           <t>[Ver. 2.28]</t>
         </is>
       </c>
-      <c r="G121" s="6" t="n">
+      <c r="G121" s="8" t="n">
         <v>46096.71458333333</v>
       </c>
-      <c r="H121" s="6" t="n">
+      <c r="H121" s="8" t="n">
         <v>46096.71458333333</v>
       </c>
-      <c r="I121" t="inlineStr"/>
+      <c r="I121" s="8" t="n"/>
       <c r="J121" t="inlineStr">
         <is>
           <t>WAPSA</t>
@@ -16768,13 +16809,13 @@
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
-      <c r="G122" s="6" t="n">
+      <c r="G122" s="8" t="n">
         <v>46097.56319444445</v>
       </c>
-      <c r="H122" s="6" t="n">
+      <c r="H122" s="8" t="n">
         <v>46097.56319444445</v>
       </c>
-      <c r="I122" s="6" t="n">
+      <c r="I122" s="8" t="n">
         <v>46097.56319444445</v>
       </c>
       <c r="J122" t="inlineStr">
@@ -16841,9 +16882,9 @@
       </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
+      <c r="G123" s="8" t="n"/>
+      <c r="H123" s="8" t="n"/>
+      <c r="I123" s="8" t="n"/>
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="n">
@@ -16896,13 +16937,13 @@
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
-      <c r="G124" s="6" t="n">
+      <c r="G124" s="8" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="H124" s="6" t="n">
+      <c r="H124" s="8" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="I124" s="6" t="n">
+      <c r="I124" s="8" t="n">
         <v>45725.79166666666</v>
       </c>
       <c r="J124" t="inlineStr">
@@ -16973,13 +17014,13 @@
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" s="6" t="n">
+      <c r="G125" s="8" t="n">
         <v>45410.79166666666</v>
       </c>
-      <c r="H125" s="6" t="n">
+      <c r="H125" s="8" t="n">
         <v>45454.79166666666</v>
       </c>
-      <c r="I125" s="6" t="n">
+      <c r="I125" s="8" t="n">
         <v>45460.79166666666</v>
       </c>
       <c r="J125" t="inlineStr">
@@ -17052,13 +17093,13 @@
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" s="6" t="n">
+      <c r="G126" s="8" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="H126" s="6" t="n">
+      <c r="H126" s="8" t="n">
         <v>45454.79166666666</v>
       </c>
-      <c r="I126" s="6" t="n">
+      <c r="I126" s="8" t="n">
         <v>45454.79166666666</v>
       </c>
       <c r="J126" t="inlineStr">
@@ -17129,13 +17170,13 @@
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" s="6" t="n">
+      <c r="G127" s="8" t="n">
         <v>45466.79166666666</v>
       </c>
-      <c r="H127" s="6" t="n">
+      <c r="H127" s="8" t="n">
         <v>45466.79166666666</v>
       </c>
-      <c r="I127" s="6" t="n">
+      <c r="I127" s="8" t="n">
         <v>45466.79166666666</v>
       </c>
       <c r="J127" t="inlineStr">
@@ -17206,13 +17247,13 @@
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
-      <c r="G128" s="6" t="n">
+      <c r="G128" s="8" t="n">
         <v>45761.79166666666</v>
       </c>
-      <c r="H128" s="6" t="n">
+      <c r="H128" s="8" t="n">
         <v>45769.79166666666</v>
       </c>
-      <c r="I128" s="6" t="n">
+      <c r="I128" s="8" t="n">
         <v>45809.79166666666</v>
       </c>
       <c r="J128" t="inlineStr">
@@ -17285,13 +17326,13 @@
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
-      <c r="G129" s="6" t="n">
+      <c r="G129" s="8" t="n">
         <v>45747.79166666666</v>
       </c>
-      <c r="H129" s="6" t="n">
+      <c r="H129" s="8" t="n">
         <v>45764.39930555555</v>
       </c>
-      <c r="I129" s="6" t="n">
+      <c r="I129" s="8" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J129" t="inlineStr">
@@ -17356,13 +17397,13 @@
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
-      <c r="G130" s="6" t="n">
+      <c r="G130" s="8" t="n">
         <v>45815.29375</v>
       </c>
-      <c r="H130" s="6" t="n">
+      <c r="H130" s="8" t="n">
         <v>45815.37708333333</v>
       </c>
-      <c r="I130" s="6" t="n">
+      <c r="I130" s="8" t="n">
         <v>45822.4375</v>
       </c>
       <c r="J130" t="inlineStr">
@@ -17433,13 +17474,13 @@
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
-      <c r="G131" s="6" t="n">
+      <c r="G131" s="8" t="n">
         <v>45813.79166666666</v>
       </c>
-      <c r="H131" s="6" t="n">
+      <c r="H131" s="8" t="n">
         <v>45818.33819444444</v>
       </c>
-      <c r="I131" s="6" t="n">
+      <c r="I131" s="8" t="n">
         <v>45832.42916666667</v>
       </c>
       <c r="J131" t="inlineStr">
@@ -17510,13 +17551,13 @@
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
-      <c r="G132" s="6" t="n">
+      <c r="G132" s="8" t="n">
         <v>45820.51458333333</v>
       </c>
-      <c r="H132" s="6" t="n">
+      <c r="H132" s="8" t="n">
         <v>45820.51458333333</v>
       </c>
-      <c r="I132" s="6" t="n">
+      <c r="I132" s="8" t="n">
         <v>45827.79166666666</v>
       </c>
       <c r="J132" t="inlineStr">
@@ -17587,13 +17628,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G133" s="6" t="n">
+      <c r="G133" s="8" t="n">
         <v>45851.79166666666</v>
       </c>
-      <c r="H133" s="6" t="n">
+      <c r="H133" s="8" t="n">
         <v>45859.42916666667</v>
       </c>
-      <c r="I133" t="inlineStr"/>
+      <c r="I133" s="8" t="n"/>
       <c r="J133" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -17662,13 +17703,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G134" s="6" t="n">
+      <c r="G134" s="8" t="n">
         <v>45856.60833333333</v>
       </c>
-      <c r="H134" s="6" t="n">
+      <c r="H134" s="8" t="n">
         <v>45856.60833333333</v>
       </c>
-      <c r="I134" s="6" t="n">
+      <c r="I134" s="8" t="n">
         <v>45859.375</v>
       </c>
       <c r="J134" t="inlineStr">
@@ -17739,13 +17780,13 @@
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
-      <c r="G135" s="6" t="n">
+      <c r="G135" s="8" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="H135" s="6" t="n">
+      <c r="H135" s="8" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="I135" s="6" t="n">
+      <c r="I135" s="8" t="n">
         <v>45460.79166666666</v>
       </c>
       <c r="J135" t="inlineStr">
@@ -17818,13 +17859,13 @@
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
-      <c r="G136" s="6" t="n">
+      <c r="G136" s="8" t="n">
         <v>45460.79166666666</v>
       </c>
-      <c r="H136" s="6" t="n">
+      <c r="H136" s="8" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="I136" s="6" t="n">
+      <c r="I136" s="8" t="n">
         <v>45490.79166666666</v>
       </c>
       <c r="J136" t="inlineStr">
@@ -17897,13 +17938,13 @@
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
-      <c r="G137" s="6" t="n">
+      <c r="G137" s="8" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="H137" s="6" t="n">
+      <c r="H137" s="8" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="I137" s="6" t="n">
+      <c r="I137" s="8" t="n">
         <v>45510.79166666666</v>
       </c>
       <c r="J137" t="inlineStr">
@@ -17976,13 +18017,13 @@
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
-      <c r="G138" s="6" t="n">
+      <c r="G138" s="8" t="n">
         <v>45475.79166666666</v>
       </c>
-      <c r="H138" s="6" t="n">
+      <c r="H138" s="8" t="n">
         <v>45475.79166666666</v>
       </c>
-      <c r="I138" s="6" t="n">
+      <c r="I138" s="8" t="n">
         <v>45475.79166666666</v>
       </c>
       <c r="J138" t="inlineStr">
@@ -18053,13 +18094,13 @@
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="G139" s="6" t="n">
+      <c r="G139" s="8" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="H139" s="6" t="n">
+      <c r="H139" s="8" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="I139" s="6" t="n">
+      <c r="I139" s="8" t="n">
         <v>45479.79166666666</v>
       </c>
       <c r="J139" t="inlineStr">
@@ -18130,13 +18171,13 @@
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" s="6" t="n">
+      <c r="G140" s="8" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="H140" s="6" t="n">
+      <c r="H140" s="8" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="I140" s="6" t="n">
+      <c r="I140" s="8" t="n">
         <v>45487.79166666666</v>
       </c>
       <c r="J140" t="inlineStr">
@@ -18207,13 +18248,13 @@
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
-      <c r="G141" s="6" t="n">
+      <c r="G141" s="8" t="n">
         <v>45496.79166666666</v>
       </c>
-      <c r="H141" s="6" t="n">
+      <c r="H141" s="8" t="n">
         <v>45496.79166666666</v>
       </c>
-      <c r="I141" s="6" t="n">
+      <c r="I141" s="8" t="n">
         <v>45496.79166666666</v>
       </c>
       <c r="J141" t="inlineStr">
@@ -18288,13 +18329,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G142" s="6" t="n">
+      <c r="G142" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H142" s="6" t="n">
+      <c r="H142" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I142" s="6" t="n">
+      <c r="I142" s="8" t="n">
         <v>45333.79166666666</v>
       </c>
       <c r="J142" t="inlineStr">
@@ -18369,13 +18410,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G143" s="6" t="n">
+      <c r="G143" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H143" s="6" t="n">
+      <c r="H143" s="8" t="n">
         <v>45334.79166666666</v>
       </c>
-      <c r="I143" s="6" t="n">
+      <c r="I143" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J143" t="inlineStr">
@@ -18450,13 +18491,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G144" s="6" t="n">
+      <c r="G144" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H144" s="6" t="n">
+      <c r="H144" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I144" s="6" t="n">
+      <c r="I144" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J144" t="inlineStr">
@@ -18531,13 +18572,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G145" s="6" t="n">
+      <c r="G145" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H145" s="6" t="n">
+      <c r="H145" s="8" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I145" s="6" t="n">
+      <c r="I145" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J145" t="inlineStr">
@@ -18612,13 +18653,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G146" s="6" t="n">
+      <c r="G146" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H146" s="6" t="n">
+      <c r="H146" s="8" t="n">
         <v>45321.79166666666</v>
       </c>
-      <c r="I146" s="6" t="n">
+      <c r="I146" s="8" t="n">
         <v>45323.79166666666</v>
       </c>
       <c r="J146" t="inlineStr">
@@ -18695,13 +18736,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G147" s="6" t="n">
+      <c r="G147" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H147" s="6" t="n">
+      <c r="H147" s="8" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I147" s="6" t="n">
+      <c r="I147" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J147" t="inlineStr">
@@ -18772,13 +18813,13 @@
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
-      <c r="G148" s="6" t="n">
+      <c r="G148" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H148" s="6" t="n">
+      <c r="H148" s="8" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I148" s="6" t="n">
+      <c r="I148" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J148" t="inlineStr">
@@ -18853,13 +18894,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G149" s="6" t="n">
+      <c r="G149" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H149" s="6" t="n">
+      <c r="H149" s="8" t="n">
         <v>45322.79166666666</v>
       </c>
-      <c r="I149" s="6" t="n">
+      <c r="I149" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J149" t="inlineStr">
@@ -18934,13 +18975,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G150" s="6" t="n">
+      <c r="G150" s="8" t="n">
         <v>45320.79166666666</v>
       </c>
-      <c r="H150" s="6" t="n">
+      <c r="H150" s="8" t="n">
         <v>45321.79166666666</v>
       </c>
-      <c r="I150" s="6" t="n">
+      <c r="I150" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J150" t="inlineStr">
@@ -19015,13 +19056,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G151" s="6" t="n">
+      <c r="G151" s="8" t="n">
         <v>45322.79166666666</v>
       </c>
-      <c r="H151" s="6" t="n">
+      <c r="H151" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I151" s="6" t="n">
+      <c r="I151" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J151" t="inlineStr">
@@ -19098,13 +19139,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G152" s="6" t="n">
+      <c r="G152" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H152" s="6" t="n">
+      <c r="H152" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I152" s="6" t="n">
+      <c r="I152" s="8" t="n">
         <v>45347.79166666666</v>
       </c>
       <c r="J152" t="inlineStr">
@@ -19181,13 +19222,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G153" s="6" t="n">
+      <c r="G153" s="8" t="n">
         <v>45326.79166666666</v>
       </c>
-      <c r="H153" s="6" t="n">
+      <c r="H153" s="8" t="n">
         <v>45326.79166666666</v>
       </c>
-      <c r="I153" s="6" t="n">
+      <c r="I153" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J153" t="inlineStr">
@@ -19268,13 +19309,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G154" s="6" t="n">
+      <c r="G154" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="H154" s="6" t="n">
+      <c r="H154" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="I154" s="6" t="n">
+      <c r="I154" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
       <c r="J154" t="inlineStr">
@@ -19349,13 +19390,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G155" s="6" t="n">
+      <c r="G155" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="H155" s="6" t="n">
+      <c r="H155" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="I155" s="6" t="n">
+      <c r="I155" s="8" t="n">
         <v>45328.79166666666</v>
       </c>
       <c r="J155" t="inlineStr">
@@ -19434,13 +19475,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G156" s="6" t="n">
+      <c r="G156" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="H156" s="6" t="n">
+      <c r="H156" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I156" s="6" t="n">
+      <c r="I156" s="8" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J156" t="inlineStr">
@@ -19511,13 +19552,13 @@
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
-      <c r="G157" s="6" t="n">
+      <c r="G157" s="8" t="n">
         <v>45333.79166666666</v>
       </c>
-      <c r="H157" s="6" t="n">
+      <c r="H157" s="8" t="n">
         <v>45333.79166666666</v>
       </c>
-      <c r="I157" s="6" t="n">
+      <c r="I157" s="8" t="n">
         <v>45340.79166666666</v>
       </c>
       <c r="J157" t="inlineStr">
@@ -19592,13 +19633,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G158" s="6" t="n">
+      <c r="G158" s="8" t="n">
         <v>45336.79166666666</v>
       </c>
-      <c r="H158" s="6" t="n">
+      <c r="H158" s="8" t="n">
         <v>45336.79166666666</v>
       </c>
-      <c r="I158" s="6" t="n">
+      <c r="I158" s="8" t="n">
         <v>45336.79166666666</v>
       </c>
       <c r="J158" t="inlineStr">
@@ -19669,13 +19710,13 @@
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
-      <c r="G159" s="6" t="n">
+      <c r="G159" s="8" t="n">
         <v>45347.79166666666</v>
       </c>
-      <c r="H159" s="6" t="n">
+      <c r="H159" s="8" t="n">
         <v>45348.79166666666</v>
       </c>
-      <c r="I159" s="6" t="n">
+      <c r="I159" s="8" t="n">
         <v>45348.79166666666</v>
       </c>
       <c r="J159" t="inlineStr">
@@ -19746,13 +19787,13 @@
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
-      <c r="G160" s="6" t="n">
+      <c r="G160" s="8" t="n">
         <v>46051.25902777778</v>
       </c>
-      <c r="H160" s="6" t="n">
+      <c r="H160" s="8" t="n">
         <v>46051.25902777778</v>
       </c>
-      <c r="I160" s="6" t="n">
+      <c r="I160" s="8" t="n">
         <v>46057.79166666666</v>
       </c>
       <c r="J160" t="inlineStr">
@@ -19819,13 +19860,13 @@
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
-      <c r="G161" s="6" t="n">
+      <c r="G161" s="8" t="n">
         <v>46059.29791666667</v>
       </c>
-      <c r="H161" s="6" t="n">
+      <c r="H161" s="8" t="n">
         <v>46059.29791666667</v>
       </c>
-      <c r="I161" s="6" t="n">
+      <c r="I161" s="8" t="n">
         <v>46062.79166666666</v>
       </c>
       <c r="J161" t="inlineStr">
@@ -19898,13 +19939,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G162" s="6" t="n">
+      <c r="G162" s="8" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="H162" s="6" t="n">
+      <c r="H162" s="8" t="n">
         <v>45670.79166666666</v>
       </c>
-      <c r="I162" s="6" t="n">
+      <c r="I162" s="8" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J162" t="inlineStr">
@@ -19979,13 +20020,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G163" s="6" t="n">
+      <c r="G163" s="8" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="H163" s="6" t="n">
+      <c r="H163" s="8" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="I163" s="6" t="n">
+      <c r="I163" s="8" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J163" t="inlineStr">
@@ -20060,13 +20101,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G164" s="6" t="n">
+      <c r="G164" s="8" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="H164" s="6" t="n">
+      <c r="H164" s="8" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="I164" s="6" t="n">
+      <c r="I164" s="8" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J164" t="inlineStr">
@@ -20141,13 +20182,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G165" s="6" t="n">
+      <c r="G165" s="8" t="n">
         <v>45674.79166666666</v>
       </c>
-      <c r="H165" s="6" t="n">
+      <c r="H165" s="8" t="n">
         <v>45674.79166666666</v>
       </c>
-      <c r="I165" s="6" t="n">
+      <c r="I165" s="8" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J165" t="inlineStr">
@@ -20222,13 +20263,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G166" s="6" t="n">
+      <c r="G166" s="8" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="H166" s="6" t="n">
+      <c r="H166" s="8" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="I166" s="6" t="n">
+      <c r="I166" s="8" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J166" t="inlineStr">
@@ -20303,13 +20344,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G167" s="6" t="n">
+      <c r="G167" s="8" t="n">
         <v>45313.79166666666</v>
       </c>
-      <c r="H167" s="6" t="n">
+      <c r="H167" s="8" t="n">
         <v>45316.79166666666</v>
       </c>
-      <c r="I167" s="6" t="n">
+      <c r="I167" s="8" t="n">
         <v>45316.79166666666</v>
       </c>
       <c r="J167" t="inlineStr">
@@ -20386,13 +20427,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G168" s="6" t="n">
+      <c r="G168" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H168" s="6" t="n">
+      <c r="H168" s="8" t="n">
         <v>45316.79166666666</v>
       </c>
-      <c r="I168" s="6" t="n">
+      <c r="I168" s="8" t="n">
         <v>45319.79166666666</v>
       </c>
       <c r="J168" t="inlineStr">
@@ -20467,13 +20508,13 @@
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
-      <c r="G169" s="6" t="n">
+      <c r="G169" s="8" t="n">
         <v>45986.79166666666</v>
       </c>
-      <c r="H169" s="6" t="n">
+      <c r="H169" s="8" t="n">
         <v>45988.79166666666</v>
       </c>
-      <c r="I169" s="6" t="n">
+      <c r="I169" s="8" t="n">
         <v>46049.79166666666</v>
       </c>
       <c r="J169" t="inlineStr">
@@ -20540,13 +20581,13 @@
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
-      <c r="G170" s="6" t="n">
+      <c r="G170" s="8" t="n">
         <v>46048.33472222222</v>
       </c>
-      <c r="H170" s="6" t="n">
+      <c r="H170" s="8" t="n">
         <v>46048.41805555556</v>
       </c>
-      <c r="I170" s="6" t="n">
+      <c r="I170" s="8" t="n">
         <v>46051.29166666666</v>
       </c>
       <c r="J170" t="inlineStr"/>
@@ -20615,13 +20656,13 @@
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
-      <c r="G171" s="6" t="n">
+      <c r="G171" s="8" t="n">
         <v>45657.79166666666</v>
       </c>
-      <c r="H171" s="6" t="n">
+      <c r="H171" s="8" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="I171" s="6" t="n">
+      <c r="I171" s="8" t="n">
         <v>45662.79166666666</v>
       </c>
       <c r="J171" t="inlineStr">
@@ -20692,13 +20733,13 @@
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
-      <c r="G172" s="6" t="n">
+      <c r="G172" s="8" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="H172" s="6" t="n">
+      <c r="H172" s="8" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="I172" s="6" t="n">
+      <c r="I172" s="8" t="n">
         <v>45683.79166666666</v>
       </c>
       <c r="J172" t="inlineStr">
@@ -20771,13 +20812,13 @@
         </is>
       </c>
       <c r="F173" t="inlineStr"/>
-      <c r="G173" s="6" t="n">
+      <c r="G173" s="8" t="n">
         <v>45662.79166666666</v>
       </c>
-      <c r="H173" s="6" t="n">
+      <c r="H173" s="8" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I173" s="6" t="n">
+      <c r="I173" s="8" t="n">
         <v>45665.79166666666</v>
       </c>
       <c r="J173" t="inlineStr">
@@ -20848,13 +20889,13 @@
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
-      <c r="G174" s="6" t="n">
+      <c r="G174" s="8" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="H174" s="6" t="n">
+      <c r="H174" s="8" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I174" s="6" t="n">
+      <c r="I174" s="8" t="n">
         <v>45683.79166666666</v>
       </c>
       <c r="J174" t="inlineStr">
@@ -20921,13 +20962,13 @@
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
-      <c r="G175" s="6" t="n">
+      <c r="G175" s="8" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="H175" s="6" t="n">
+      <c r="H175" s="8" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="I175" s="6" t="n">
+      <c r="I175" s="8" t="n">
         <v>45694.79166666666</v>
       </c>
       <c r="J175" t="inlineStr">
@@ -20998,13 +21039,13 @@
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
-      <c r="G176" s="6" t="n">
+      <c r="G176" s="8" t="n">
         <v>45682.79166666666</v>
       </c>
-      <c r="H176" s="6" t="n">
+      <c r="H176" s="8" t="n">
         <v>45683.79166666666</v>
       </c>
-      <c r="I176" s="6" t="n">
+      <c r="I176" s="8" t="n">
         <v>45694.79166666666</v>
       </c>
       <c r="J176" t="inlineStr">
@@ -21077,13 +21118,13 @@
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
-      <c r="G177" s="6" t="n">
+      <c r="G177" s="8" t="n">
         <v>45687.79166666666</v>
       </c>
-      <c r="H177" s="6" t="n">
+      <c r="H177" s="8" t="n">
         <v>45687.79166666666</v>
       </c>
-      <c r="I177" s="6" t="n">
+      <c r="I177" s="8" t="n">
         <v>45688.79166666666</v>
       </c>
       <c r="J177" t="inlineStr">
@@ -21156,13 +21197,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G178" s="6" t="n">
+      <c r="G178" s="8" t="n">
         <v>45963.79166666666</v>
       </c>
-      <c r="H178" s="6" t="n">
+      <c r="H178" s="8" t="n">
         <v>45987.43333333333</v>
       </c>
-      <c r="I178" t="inlineStr"/>
+      <c r="I178" s="8" t="n"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21235,13 +21276,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G179" s="6" t="n">
+      <c r="G179" s="8" t="n">
         <v>45944.79166666666</v>
       </c>
-      <c r="H179" s="6" t="n">
+      <c r="H179" s="8" t="n">
         <v>45951.79166666666</v>
       </c>
-      <c r="I179" t="inlineStr"/>
+      <c r="I179" s="8" t="n"/>
       <c r="J179" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21310,13 +21351,13 @@
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
-      <c r="G180" s="6" t="n">
+      <c r="G180" s="8" t="n">
         <v>45963.79166666666</v>
       </c>
-      <c r="H180" s="6" t="n">
+      <c r="H180" s="8" t="n">
         <v>45979.79166666666</v>
       </c>
-      <c r="I180" s="6" t="n">
+      <c r="I180" s="8" t="n">
         <v>46008.79166666666</v>
       </c>
       <c r="J180" t="inlineStr">
@@ -21387,13 +21428,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G181" s="6" t="n">
+      <c r="G181" s="8" t="n">
         <v>45908.79166666666</v>
       </c>
-      <c r="H181" s="6" t="n">
+      <c r="H181" s="8" t="n">
         <v>45930.79166666666</v>
       </c>
-      <c r="I181" t="inlineStr"/>
+      <c r="I181" s="8" t="n"/>
       <c r="J181" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21462,13 +21503,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G182" s="6" t="n">
+      <c r="G182" s="8" t="n">
         <v>45936.79166666666</v>
       </c>
-      <c r="H182" s="6" t="n">
+      <c r="H182" s="8" t="n">
         <v>45950.79166666666</v>
       </c>
-      <c r="I182" t="inlineStr"/>
+      <c r="I182" s="8" t="n"/>
       <c r="J182" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21533,13 +21574,13 @@
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
-      <c r="G183" s="6" t="n">
+      <c r="G183" s="8" t="n">
         <v>45995.79166666666</v>
       </c>
-      <c r="H183" s="6" t="n">
+      <c r="H183" s="8" t="n">
         <v>46006.29166666666</v>
       </c>
-      <c r="I183" t="inlineStr"/>
+      <c r="I183" s="8" t="n"/>
       <c r="J183" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21608,13 +21649,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G184" s="6" t="n">
+      <c r="G184" s="8" t="n">
         <v>45970.79166666666</v>
       </c>
-      <c r="H184" s="6" t="n">
+      <c r="H184" s="8" t="n">
         <v>45974.51111111111</v>
       </c>
-      <c r="I184" t="inlineStr"/>
+      <c r="I184" s="8" t="n"/>
       <c r="J184" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21683,13 +21724,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G185" s="6" t="n">
+      <c r="G185" s="8" t="n">
         <v>45981.79166666666</v>
       </c>
-      <c r="H185" s="6" t="n">
+      <c r="H185" s="8" t="n">
         <v>46006.43541666667</v>
       </c>
-      <c r="I185" t="inlineStr"/>
+      <c r="I185" s="8" t="n"/>
       <c r="J185" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21754,13 +21795,13 @@
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
-      <c r="G186" s="6" t="n">
+      <c r="G186" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H186" s="6" t="n">
+      <c r="H186" s="8" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I186" s="6" t="n">
+      <c r="I186" s="8" t="n">
         <v>45652.79166666666</v>
       </c>
       <c r="J186" t="inlineStr">
@@ -21833,13 +21874,13 @@
         </is>
       </c>
       <c r="F187" t="inlineStr"/>
-      <c r="G187" s="6" t="n">
+      <c r="G187" s="8" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="H187" s="6" t="n">
+      <c r="H187" s="8" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="I187" s="6" t="n">
+      <c r="I187" s="8" t="n">
         <v>45651.79166666666</v>
       </c>
       <c r="J187" t="inlineStr">
@@ -21916,13 +21957,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G188" s="6" t="n">
+      <c r="G188" s="8" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="H188" s="6" t="n">
+      <c r="H188" s="8" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="I188" s="6" t="n">
+      <c r="I188" s="8" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J188" t="inlineStr">
@@ -21997,13 +22038,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G189" s="6" t="n">
+      <c r="G189" s="8" t="n">
         <v>45820.79166666666</v>
       </c>
-      <c r="H189" s="6" t="n">
+      <c r="H189" s="8" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I189" t="inlineStr"/>
+      <c r="I189" s="8" t="n"/>
       <c r="J189" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -22076,13 +22117,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G190" s="6" t="n">
+      <c r="G190" s="8" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="H190" s="6" t="n">
+      <c r="H190" s="8" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="I190" s="6" t="n">
+      <c r="I190" s="8" t="n">
         <v>45481.79166666666</v>
       </c>
       <c r="J190" t="inlineStr">
@@ -22153,13 +22194,13 @@
         </is>
       </c>
       <c r="F191" t="inlineStr"/>
-      <c r="G191" s="6" t="n">
+      <c r="G191" s="8" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="H191" s="6" t="n">
+      <c r="H191" s="8" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="I191" s="6" t="n">
+      <c r="I191" s="8" t="n">
         <v>45508.79166666666</v>
       </c>
       <c r="J191" t="inlineStr">
@@ -22232,13 +22273,13 @@
         </is>
       </c>
       <c r="F192" t="inlineStr"/>
-      <c r="G192" s="6" t="n">
+      <c r="G192" s="8" t="n">
         <v>45505.79166666666</v>
       </c>
-      <c r="H192" s="6" t="n">
+      <c r="H192" s="8" t="n">
         <v>45505.79166666666</v>
       </c>
-      <c r="I192" s="6" t="n">
+      <c r="I192" s="8" t="n">
         <v>45525.79166666666</v>
       </c>
       <c r="J192" t="inlineStr">
@@ -22311,13 +22352,13 @@
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
-      <c r="G193" s="6" t="n">
+      <c r="G193" s="8" t="n">
         <v>45526.79166666666</v>
       </c>
-      <c r="H193" s="6" t="n">
+      <c r="H193" s="8" t="n">
         <v>45529.79166666666</v>
       </c>
-      <c r="I193" s="6" t="n">
+      <c r="I193" s="8" t="n">
         <v>45529.79166666666</v>
       </c>
       <c r="J193" t="inlineStr">
@@ -22388,13 +22429,13 @@
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
-      <c r="G194" s="6" t="n">
+      <c r="G194" s="8" t="n">
         <v>45528.79166666666</v>
       </c>
-      <c r="H194" s="6" t="n">
+      <c r="H194" s="8" t="n">
         <v>45528.79166666666</v>
       </c>
-      <c r="I194" s="6" t="n">
+      <c r="I194" s="8" t="n">
         <v>45528.79166666666</v>
       </c>
       <c r="J194" t="inlineStr">
@@ -22465,13 +22506,13 @@
         </is>
       </c>
       <c r="F195" t="inlineStr"/>
-      <c r="G195" s="6" t="n">
+      <c r="G195" s="8" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="H195" s="6" t="n">
+      <c r="H195" s="8" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="I195" s="6" t="n">
+      <c r="I195" s="8" t="n">
         <v>45397.79166666666</v>
       </c>
       <c r="J195" t="inlineStr">
@@ -22544,13 +22585,13 @@
         </is>
       </c>
       <c r="F196" t="inlineStr"/>
-      <c r="G196" s="6" t="n">
+      <c r="G196" s="8" t="n">
         <v>45392.79166666666</v>
       </c>
-      <c r="H196" s="6" t="n">
+      <c r="H196" s="8" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="I196" s="6" t="n">
+      <c r="I196" s="8" t="n">
         <v>45404.79166666666</v>
       </c>
       <c r="J196" t="inlineStr">
@@ -22623,13 +22664,13 @@
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
-      <c r="G197" s="6" t="n">
+      <c r="G197" s="8" t="n">
         <v>45397.79166666666</v>
       </c>
-      <c r="H197" s="6" t="n">
+      <c r="H197" s="8" t="n">
         <v>45397.79166666666</v>
       </c>
-      <c r="I197" s="6" t="n">
+      <c r="I197" s="8" t="n">
         <v>45404.79166666666</v>
       </c>
       <c r="J197" t="inlineStr">
@@ -22702,13 +22743,13 @@
         </is>
       </c>
       <c r="F198" t="inlineStr"/>
-      <c r="G198" s="6" t="n">
+      <c r="G198" s="8" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="H198" s="6" t="n">
+      <c r="H198" s="8" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="I198" s="6" t="n">
+      <c r="I198" s="8" t="n">
         <v>45413.79166666666</v>
       </c>
       <c r="J198" t="inlineStr">
@@ -22779,13 +22820,13 @@
         </is>
       </c>
       <c r="F199" t="inlineStr"/>
-      <c r="G199" s="6" t="n">
+      <c r="G199" s="8" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="H199" s="6" t="n">
+      <c r="H199" s="8" t="n">
         <v>45413.79166666666</v>
       </c>
-      <c r="I199" s="6" t="n">
+      <c r="I199" s="8" t="n">
         <v>45413.79166666666</v>
       </c>
       <c r="J199" t="inlineStr">
@@ -22858,13 +22899,13 @@
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
-      <c r="G200" s="6" t="n">
+      <c r="G200" s="8" t="n">
         <v>45693.79166666666</v>
       </c>
-      <c r="H200" s="6" t="n">
+      <c r="H200" s="8" t="n">
         <v>45704.79166666666</v>
       </c>
-      <c r="I200" s="6" t="n">
+      <c r="I200" s="8" t="n">
         <v>45755.44861111111</v>
       </c>
       <c r="J200" t="inlineStr">
@@ -22935,13 +22976,13 @@
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
-      <c r="G201" s="6" t="n">
+      <c r="G201" s="8" t="n">
         <v>45711.79166666666</v>
       </c>
-      <c r="H201" s="6" t="n">
+      <c r="H201" s="8" t="n">
         <v>45712.79166666666</v>
       </c>
-      <c r="I201" s="6" t="n">
+      <c r="I201" s="8" t="n">
         <v>45755.44861111111</v>
       </c>
       <c r="J201" t="inlineStr">
@@ -23016,13 +23057,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G202" s="6" t="n">
+      <c r="G202" s="8" t="n">
         <v>45768.79166666666</v>
       </c>
-      <c r="H202" s="6" t="n">
+      <c r="H202" s="8" t="n">
         <v>45770.79166666666</v>
       </c>
-      <c r="I202" s="6" t="n">
+      <c r="I202" s="8" t="n">
         <v>45771.79166666666</v>
       </c>
       <c r="J202" t="inlineStr">
@@ -23093,13 +23134,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G203" s="6" t="n">
+      <c r="G203" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H203" s="6" t="n">
+      <c r="H203" s="8" t="n">
         <v>45341.79166666666</v>
       </c>
-      <c r="I203" s="6" t="n">
+      <c r="I203" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J203" t="inlineStr">
@@ -23174,13 +23215,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G204" s="6" t="n">
+      <c r="G204" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H204" s="6" t="n">
+      <c r="H204" s="8" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I204" s="6" t="n">
+      <c r="I204" s="8" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J204" t="inlineStr">
@@ -23255,13 +23296,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G205" s="6" t="n">
+      <c r="G205" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H205" s="6" t="n">
+      <c r="H205" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I205" s="6" t="n">
+      <c r="I205" s="8" t="n">
         <v>45375.79166666666</v>
       </c>
       <c r="J205" t="inlineStr">
@@ -23336,13 +23377,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G206" s="6" t="n">
+      <c r="G206" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H206" s="6" t="n">
+      <c r="H206" s="8" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I206" s="6" t="n">
+      <c r="I206" s="8" t="n">
         <v>45375.79166666666</v>
       </c>
       <c r="J206" t="inlineStr">
@@ -23417,13 +23458,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G207" s="6" t="n">
+      <c r="G207" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H207" s="6" t="n">
+      <c r="H207" s="8" t="n">
         <v>45361.79166666666</v>
       </c>
-      <c r="I207" s="6" t="n">
+      <c r="I207" s="8" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J207" t="inlineStr">
@@ -23498,13 +23539,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G208" s="6" t="n">
+      <c r="G208" s="8" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H208" s="6" t="n">
+      <c r="H208" s="8" t="n">
         <v>45375.79166666666</v>
       </c>
-      <c r="I208" s="6" t="n">
+      <c r="I208" s="8" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J208" t="inlineStr">
@@ -23551,6 +23592,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Corregir colores del encabezado en data.xlsx
Fill y fuente usaban alpha 00 (transparente), dejando los titulos invisibles.
Corregido a FF106EBE (azul) y FFFFFFFF (blanco opaco).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +77,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +99,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00106EBE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF106EBE"/>
       </patternFill>
     </fill>
   </fills>
@@ -124,7 +134,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -146,6 +156,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7241,97 +7257,97 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Work Item Type</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>Iteration Path</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Estados</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="10" t="inlineStr">
         <is>
           <t>Finish Date</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>Finish Date Chinalco</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="10" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="10" t="inlineStr">
         <is>
           <t>Ticket Chinalco</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="10" t="inlineStr">
         <is>
           <t>Ticket SyC</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>Tipo Caso</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
         <is>
           <t>Tipo Evento</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="Q1" s="10" t="inlineStr">
         <is>
           <t>Tipo Estabilización</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="R1" s="10" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
+      <c r="S1" s="10" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>

</xml_diff>

<commit_message>
Usar plantilla como base para preservar formato del encabezado
Copia el archivo de referencia como base y re-aplica el fill/font
con copy() para garantizar azul opaco en todos los encabezados.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,16 +73,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -94,11 +88,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF106EBE"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00106EBE"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,7 +123,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,17 +140,10 @@
     <xf numFmtId="22" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7233,121 +7215,121 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S208"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="21.140625" defaultRowHeight="15"/>
   <cols>
     <col width="4.14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="77" customWidth="1" min="3" max="3"/>
     <col width="40.57" customWidth="1" min="4" max="4"/>
     <col width="19.57" customWidth="1" min="5" max="5"/>
     <col width="15.43" customWidth="1" min="6" max="6"/>
-    <col width="17.71" customWidth="1" min="7" max="7"/>
+    <col width="17.71" bestFit="1" customWidth="1" min="7" max="8"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15.71" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="9.289999999999999" customWidth="1" min="11" max="11"/>
-    <col width="17.71" customWidth="1" min="12" max="12"/>
-    <col width="47.71" customWidth="1" min="13" max="13"/>
-    <col width="255.71" customWidth="1" min="14" max="14"/>
+    <col width="15.71" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="13" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="9.289999999999999" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="17.71" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="47.71" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="255.71" bestFit="1" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="35.43" customWidth="1" min="16" max="16"/>
+    <col width="35.43" bestFit="1" customWidth="1" min="16" max="16"/>
     <col width="25" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="24.71" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Work Item Type</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Iteration Path</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Estados</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Finish Date</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Finish Date Chinalco</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Aplicación</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Ticket Chinalco</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Ticket SyC</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Tipo Caso</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Tipo Evento</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>Tipo Estabilización</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
@@ -7378,13 +7360,13 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="7" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="7" t="n">
         <v>45914.79166666666</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="7" t="n">
         <v>46019.79166666666</v>
       </c>
       <c r="J2" t="inlineStr">
@@ -7455,13 +7437,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="7" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -7532,9 +7514,9 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7599,9 +7581,9 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7666,9 +7648,9 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -7733,11 +7715,11 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="7" t="n">
         <v>45391.79166666666</v>
       </c>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -7806,13 +7788,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="7" t="n">
         <v>45810.79166666666</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="7" t="n">
         <v>45873.79166666666</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="7" t="n">
         <v>45937.57847222222</v>
       </c>
       <c r="J8" t="inlineStr">
@@ -7887,13 +7869,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="7" t="n">
         <v>45863.71805555555</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="7" t="n">
         <v>45863.71805555555</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="7" t="n">
         <v>45901.26458333333</v>
       </c>
       <c r="J9" t="inlineStr">
@@ -7968,13 +7950,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="7" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="7" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="7" t="n">
         <v>45530.79166666666</v>
       </c>
       <c r="J10" t="inlineStr">
@@ -8051,13 +8033,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="7" t="n">
         <v>45544.79166666666</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="7" t="n">
         <v>45544.79166666666</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J11" t="inlineStr">
@@ -8134,13 +8116,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="7" t="n">
         <v>45933.35277777778</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="7" t="n">
         <v>45937.575</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="7" t="n">
         <v>45959.20069444444</v>
       </c>
       <c r="J12" t="inlineStr">
@@ -8215,13 +8197,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="7" t="n">
         <v>45937.58055555556</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="7" t="n">
         <v>45937.58055555556</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="7" t="n">
         <v>45959.20069444444</v>
       </c>
       <c r="J13" t="inlineStr">
@@ -8296,13 +8278,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="7" t="n">
         <v>45414.79166666666</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="7" t="n">
         <v>45431.79166666666</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="7" t="n">
         <v>45426.79166666666</v>
       </c>
       <c r="J14" t="inlineStr">
@@ -8377,13 +8359,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="7" t="n">
         <v>45414.79166666666</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="7" t="n">
         <v>45440.79166666666</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J15" t="inlineStr">
@@ -8458,13 +8440,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="7" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J16" t="inlineStr">
@@ -8542,11 +8524,11 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="7" t="n">
         <v>46073.42986111111</v>
       </c>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
@@ -8615,13 +8597,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="7" t="n">
         <v>45704.79166666666</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="7" t="n">
         <v>45715.79166666666</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="7" t="n">
         <v>45728.79166666666</v>
       </c>
       <c r="J18" t="inlineStr">
@@ -8696,13 +8678,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="7" t="n">
         <v>45771.79166666666</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="7" t="n">
         <v>45774.79166666666</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="7" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J19" t="inlineStr">
@@ -8777,13 +8759,13 @@
           <t>[Ver. 2.23]</t>
         </is>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="7" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="7" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="7" t="n">
         <v>45832.42916666667</v>
       </c>
       <c r="J20" t="inlineStr">
@@ -8858,13 +8840,13 @@
           <t>[Ver 4.0]</t>
         </is>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="7" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="7" t="n">
         <v>45819.36388888889</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="7" t="n">
         <v>45827.79166666666</v>
       </c>
       <c r="J21" t="inlineStr">
@@ -8939,13 +8921,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="7" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="7" t="n">
         <v>45354.79166666666</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I22" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J22" t="inlineStr">
@@ -9036,13 +9018,13 @@
           <t>[Ver.2.4]</t>
         </is>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G23" s="7" t="n">
         <v>45337.79166666666</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="7" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="7" t="n">
         <v>45343.79166666666</v>
       </c>
       <c r="J23" t="inlineStr">
@@ -9113,13 +9095,13 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="7" t="n">
         <v>46019.79166666666</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H24" s="7" t="n">
         <v>46022.65347222222</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="7" t="n">
         <v>46045.65347222222</v>
       </c>
       <c r="J24" t="inlineStr">
@@ -9192,13 +9174,13 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="7" t="n">
         <v>46019.79166666666</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="7" t="n">
         <v>46021.79166666666</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="7" t="n">
         <v>46045.65555555555</v>
       </c>
       <c r="J25" t="inlineStr">
@@ -9275,13 +9257,13 @@
           <t>v2.25.3</t>
         </is>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="7" t="n">
         <v>45988.79166666666</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="7" t="n">
         <v>45992.59097222222</v>
       </c>
-      <c r="I26" s="8" t="n"/>
+      <c r="I26" s="7" t="n"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -9342,13 +9324,13 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" s="8" t="n">
+      <c r="G27" s="7" t="n">
         <v>45992.42916666667</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="7" t="n">
         <v>45991.79166666666</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="7" t="n">
         <v>45995.79166666666</v>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -9419,13 +9401,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I28" s="8" t="n">
+      <c r="I28" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J28" t="inlineStr">
@@ -9502,13 +9484,13 @@
           <t>[Ver. 2.20]</t>
         </is>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="7" t="n">
         <v>45665.79166666666</v>
       </c>
       <c r="J29" t="inlineStr">
@@ -9583,13 +9565,13 @@
           <t>[Ver. 1.1]</t>
         </is>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="7" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="H30" s="8" t="n">
+      <c r="H30" s="7" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="I30" s="8" t="n">
+      <c r="I30" s="7" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J30" t="inlineStr">
@@ -9660,13 +9642,13 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="7" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="H31" s="7" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="I31" s="8" t="n">
+      <c r="I31" s="7" t="n">
         <v>45550.79166666666</v>
       </c>
       <c r="J31" t="inlineStr">
@@ -9739,13 +9721,13 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="7" t="n">
         <v>45427.79166666666</v>
       </c>
-      <c r="H32" s="8" t="n">
+      <c r="H32" s="7" t="n">
         <v>45439.79166666666</v>
       </c>
-      <c r="I32" s="8" t="n">
+      <c r="I32" s="7" t="n">
         <v>45440.79166666666</v>
       </c>
       <c r="J32" t="inlineStr">
@@ -9818,13 +9800,13 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="7" t="n">
         <v>45348.79166666666</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="7" t="n">
         <v>45354.79166666666</v>
       </c>
       <c r="J33" t="inlineStr">
@@ -9895,13 +9877,13 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I34" s="8" t="n">
+      <c r="I34" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
       <c r="J34" t="inlineStr">
@@ -9974,13 +9956,13 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="7" t="n">
         <v>45383.79166666666</v>
       </c>
       <c r="J35" t="inlineStr">
@@ -10053,13 +10035,13 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="7" t="n">
         <v>45396.79166666666</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="7" t="n">
         <v>45415.79166666666</v>
       </c>
-      <c r="I36" s="8" t="n">
+      <c r="I36" s="7" t="n">
         <v>45415.79166666666</v>
       </c>
       <c r="J36" t="inlineStr">
@@ -10136,13 +10118,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="7" t="n">
         <v>45911.30347222222</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
-      <c r="I37" s="8" t="n">
+      <c r="I37" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J37" t="inlineStr">
@@ -10213,9 +10195,9 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" s="8" t="n"/>
-      <c r="H38" s="8" t="n"/>
-      <c r="I38" s="8" t="n"/>
+      <c r="G38" s="7" t="n"/>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10284,13 +10266,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="7" t="n">
         <v>45930.79166666666</v>
       </c>
-      <c r="H39" s="8" t="n">
+      <c r="H39" s="7" t="n">
         <v>45937.45138888889</v>
       </c>
-      <c r="I39" s="8" t="n">
+      <c r="I39" s="7" t="n">
         <v>45937.57986111111</v>
       </c>
       <c r="J39" t="inlineStr">
@@ -10361,9 +10343,9 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" s="8" t="n"/>
-      <c r="H40" s="8" t="n"/>
-      <c r="I40" s="8" t="n"/>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="7" t="n"/>
+      <c r="I40" s="7" t="n"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10432,11 +10414,11 @@
           <t>[Ver. 2.27]; [Ver. 2.28]</t>
         </is>
       </c>
-      <c r="G41" s="8" t="n">
+      <c r="G41" s="7" t="n">
         <v>45991.79166666666</v>
       </c>
-      <c r="H41" s="8" t="n"/>
-      <c r="I41" s="8" t="n"/>
+      <c r="H41" s="7" t="n"/>
+      <c r="I41" s="7" t="n"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10505,13 +10487,13 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" s="8" t="n">
+      <c r="G42" s="7" t="n">
         <v>45931.79166666666</v>
       </c>
-      <c r="H42" s="8" t="n">
+      <c r="H42" s="7" t="n">
         <v>46008.79166666666</v>
       </c>
-      <c r="I42" s="8" t="n">
+      <c r="I42" s="7" t="n">
         <v>46008.79166666666</v>
       </c>
       <c r="J42" t="inlineStr">
@@ -10586,13 +10568,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G43" s="8" t="n">
+      <c r="G43" s="7" t="n">
         <v>45854.72638888889</v>
       </c>
-      <c r="H43" s="8" t="n">
+      <c r="H43" s="7" t="n">
         <v>45854.72638888889</v>
       </c>
-      <c r="I43" s="8" t="n"/>
+      <c r="I43" s="7" t="n"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10665,13 +10647,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G44" s="8" t="n">
+      <c r="G44" s="7" t="n">
         <v>45417.79166666666</v>
       </c>
-      <c r="H44" s="8" t="n">
+      <c r="H44" s="7" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="I44" s="8" t="n">
+      <c r="I44" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J44" t="inlineStr">
@@ -10746,13 +10728,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G45" s="8" t="n">
+      <c r="G45" s="7" t="n">
         <v>45426.79166666666</v>
       </c>
-      <c r="H45" s="8" t="n">
+      <c r="H45" s="7" t="n">
         <v>45476.79166666666</v>
       </c>
-      <c r="I45" s="8" t="n">
+      <c r="I45" s="7" t="n">
         <v>45538.79166666666</v>
       </c>
       <c r="J45" t="inlineStr">
@@ -10827,13 +10809,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G46" s="8" t="n">
+      <c r="G46" s="7" t="n">
         <v>45445.79166666666</v>
       </c>
-      <c r="H46" s="8" t="n">
+      <c r="H46" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I46" s="8" t="n">
+      <c r="I46" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J46" t="inlineStr">
@@ -10908,13 +10890,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G47" s="8" t="n">
+      <c r="G47" s="7" t="n">
         <v>45382.79166666666</v>
       </c>
-      <c r="H47" s="8" t="n">
+      <c r="H47" s="7" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="I47" s="8" t="n">
+      <c r="I47" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J47" t="inlineStr">
@@ -10985,13 +10967,13 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" s="8" t="n">
+      <c r="G48" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
-      <c r="H48" s="8" t="n">
+      <c r="H48" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I48" s="8" t="n">
+      <c r="I48" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J48" t="inlineStr">
@@ -11062,13 +11044,13 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" s="8" t="n">
+      <c r="G49" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
-      <c r="H49" s="8" t="n">
+      <c r="H49" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I49" s="8" t="n">
+      <c r="I49" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
       <c r="J49" t="inlineStr">
@@ -11143,11 +11125,11 @@
           <t>[Ver. 1.3]</t>
         </is>
       </c>
-      <c r="G50" s="8" t="n">
+      <c r="G50" s="7" t="n">
         <v>45446.79166666666</v>
       </c>
-      <c r="H50" s="8" t="n"/>
-      <c r="I50" s="8" t="n"/>
+      <c r="H50" s="7" t="n"/>
+      <c r="I50" s="7" t="n"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>Wapsa ES</t>
@@ -11220,13 +11202,13 @@
           <t>[Ver. 1.3]</t>
         </is>
       </c>
-      <c r="G51" s="8" t="n">
+      <c r="G51" s="7" t="n">
         <v>45420.79166666666</v>
       </c>
-      <c r="H51" s="8" t="n">
+      <c r="H51" s="7" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="I51" s="8" t="n">
+      <c r="I51" s="7" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J51" t="inlineStr">
@@ -11301,13 +11283,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G52" s="8" t="n">
+      <c r="G52" s="7" t="n">
         <v>45439.79166666666</v>
       </c>
-      <c r="H52" s="8" t="n">
+      <c r="H52" s="7" t="n">
         <v>45482.79166666666</v>
       </c>
-      <c r="I52" s="8" t="n">
+      <c r="I52" s="7" t="n">
         <v>45489.79166666666</v>
       </c>
       <c r="J52" t="inlineStr">
@@ -11382,13 +11364,13 @@
           <t>[Ver. 1.1]</t>
         </is>
       </c>
-      <c r="G53" s="8" t="n">
+      <c r="G53" s="7" t="n">
         <v>45420.79166666666</v>
       </c>
-      <c r="H53" s="8" t="n">
+      <c r="H53" s="7" t="n">
         <v>45421.79166666666</v>
       </c>
-      <c r="I53" s="8" t="n">
+      <c r="I53" s="7" t="n">
         <v>45511.79166666666</v>
       </c>
       <c r="J53" t="inlineStr">
@@ -11463,13 +11445,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G54" s="8" t="n">
+      <c r="G54" s="7" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="H54" s="8" t="n">
+      <c r="H54" s="7" t="n">
         <v>45901.79166666666</v>
       </c>
-      <c r="I54" s="8" t="n">
+      <c r="I54" s="7" t="n">
         <v>45937.57847222222</v>
       </c>
       <c r="J54" t="inlineStr">
@@ -11544,13 +11526,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G55" s="8" t="n">
+      <c r="G55" s="7" t="n">
         <v>45874.79166666666</v>
       </c>
-      <c r="H55" s="8" t="n">
+      <c r="H55" s="7" t="n">
         <v>45900.79166666666</v>
       </c>
-      <c r="I55" s="8" t="n">
+      <c r="I55" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J55" t="inlineStr">
@@ -11625,13 +11607,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G56" s="8" t="n">
+      <c r="G56" s="7" t="n">
         <v>45739.79166666666</v>
       </c>
-      <c r="H56" s="8" t="n">
+      <c r="H56" s="7" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I56" s="8" t="n">
+      <c r="I56" s="7" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J56" t="inlineStr">
@@ -11706,13 +11688,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G57" s="8" t="n">
+      <c r="G57" s="7" t="n">
         <v>45724.79166666666</v>
       </c>
-      <c r="H57" s="8" t="n">
+      <c r="H57" s="7" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="I57" s="8" t="n">
+      <c r="I57" s="7" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J57" t="inlineStr">
@@ -11783,13 +11765,13 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" s="8" t="n">
+      <c r="G58" s="7" t="n">
         <v>46022.79166666666</v>
       </c>
-      <c r="H58" s="8" t="n">
+      <c r="H58" s="7" t="n">
         <v>46052.79166666666</v>
       </c>
-      <c r="I58" s="8" t="n">
+      <c r="I58" s="7" t="n">
         <v>46052.79166666666</v>
       </c>
       <c r="J58" t="inlineStr">
@@ -11860,13 +11842,13 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" s="8" t="n">
+      <c r="G59" s="7" t="n">
         <v>45987.11875</v>
       </c>
-      <c r="H59" s="8" t="n">
+      <c r="H59" s="7" t="n">
         <v>45996.11875</v>
       </c>
-      <c r="I59" s="8" t="n">
+      <c r="I59" s="7" t="n">
         <v>45996.11875</v>
       </c>
       <c r="J59" t="inlineStr">
@@ -11941,13 +11923,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G60" s="8" t="n">
+      <c r="G60" s="7" t="n">
         <v>45762.79166666666</v>
       </c>
-      <c r="H60" s="8" t="n">
+      <c r="H60" s="7" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I60" s="8" t="n"/>
+      <c r="I60" s="7" t="n"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>WAPSA web</t>
@@ -12020,13 +12002,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G61" s="8" t="n">
+      <c r="G61" s="7" t="n">
         <v>45739.79166666666</v>
       </c>
-      <c r="H61" s="8" t="n">
+      <c r="H61" s="7" t="n">
         <v>45822.79166666666</v>
       </c>
-      <c r="I61" s="8" t="n"/>
+      <c r="I61" s="7" t="n"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -12099,13 +12081,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G62" s="8" t="n">
+      <c r="G62" s="7" t="n">
         <v>45713.79166666666</v>
       </c>
-      <c r="H62" s="8" t="n">
+      <c r="H62" s="7" t="n">
         <v>45726.79166666666</v>
       </c>
-      <c r="I62" s="8" t="n">
+      <c r="I62" s="7" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J62" t="inlineStr">
@@ -12176,13 +12158,13 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" s="8" t="n">
+      <c r="G63" s="7" t="n">
         <v>45864.14652777778</v>
       </c>
-      <c r="H63" s="8" t="n">
+      <c r="H63" s="7" t="n">
         <v>45873.79166666666</v>
       </c>
-      <c r="I63" s="8" t="n">
+      <c r="I63" s="7" t="n">
         <v>45873.79166666666</v>
       </c>
       <c r="J63" t="inlineStr">
@@ -12249,13 +12231,13 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" s="8" t="n">
+      <c r="G64" s="7" t="n">
         <v>45886.79166666666</v>
       </c>
-      <c r="H64" s="8" t="n">
+      <c r="H64" s="7" t="n">
         <v>45931.79166666666</v>
       </c>
-      <c r="I64" s="8" t="n">
+      <c r="I64" s="7" t="n">
         <v>45930.79166666666</v>
       </c>
       <c r="J64" t="inlineStr">
@@ -12322,13 +12304,13 @@
           <t>[Ver. 2.24.1]</t>
         </is>
       </c>
-      <c r="G65" s="8" t="n">
+      <c r="G65" s="7" t="n">
         <v>45926.29791666667</v>
       </c>
-      <c r="H65" s="8" t="n">
+      <c r="H65" s="7" t="n">
         <v>45927.79166666666</v>
       </c>
-      <c r="I65" s="8" t="n">
+      <c r="I65" s="7" t="n">
         <v>45959.2</v>
       </c>
       <c r="J65" t="inlineStr">
@@ -12403,13 +12385,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G66" s="8" t="n">
+      <c r="G66" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="H66" s="8" t="n">
+      <c r="H66" s="7" t="n">
         <v>45441.79166666666</v>
       </c>
-      <c r="I66" s="8" t="n">
+      <c r="I66" s="7" t="n">
         <v>45522.79166666666</v>
       </c>
       <c r="J66" t="inlineStr">
@@ -12480,13 +12462,13 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" s="8" t="n">
+      <c r="G67" s="7" t="n">
         <v>45517.79166666666</v>
       </c>
-      <c r="H67" s="8" t="n">
+      <c r="H67" s="7" t="n">
         <v>45517.79166666666</v>
       </c>
-      <c r="I67" s="8" t="n">
+      <c r="I67" s="7" t="n">
         <v>45538.79166666666</v>
       </c>
       <c r="J67" t="inlineStr">
@@ -12559,13 +12541,13 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" s="8" t="n">
+      <c r="G68" s="7" t="n">
         <v>45546.79166666666</v>
       </c>
-      <c r="H68" s="8" t="n">
+      <c r="H68" s="7" t="n">
         <v>45546.79166666666</v>
       </c>
-      <c r="I68" s="8" t="n">
+      <c r="I68" s="7" t="n">
         <v>45574.79166666666</v>
       </c>
       <c r="J68" t="inlineStr">
@@ -12638,13 +12620,13 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" s="8" t="n">
+      <c r="G69" s="7" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="H69" s="8" t="n">
+      <c r="H69" s="7" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="I69" s="8" t="n">
+      <c r="I69" s="7" t="n">
         <v>45540.79166666666</v>
       </c>
       <c r="J69" t="inlineStr">
@@ -12715,13 +12697,13 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" s="8" t="n">
+      <c r="G70" s="7" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="H70" s="8" t="n">
+      <c r="H70" s="7" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="I70" s="8" t="n">
+      <c r="I70" s="7" t="n">
         <v>45558.79166666666</v>
       </c>
       <c r="J70" t="inlineStr">
@@ -12796,13 +12778,13 @@
           <t>[Ver 2.25]; [Ver 4.1]</t>
         </is>
       </c>
-      <c r="G71" s="8" t="n">
+      <c r="G71" s="7" t="n">
         <v>45578.79166666666</v>
       </c>
-      <c r="H71" s="8" t="n">
+      <c r="H71" s="7" t="n">
         <v>45904.26666666667</v>
       </c>
-      <c r="I71" s="8" t="n">
+      <c r="I71" s="7" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J71" t="inlineStr">
@@ -12877,13 +12859,13 @@
           <t>[Ver 4.1]</t>
         </is>
       </c>
-      <c r="G72" s="8" t="n">
+      <c r="G72" s="7" t="n">
         <v>45643.79166666666</v>
       </c>
-      <c r="H72" s="8" t="n">
+      <c r="H72" s="7" t="n">
         <v>45904.26111111111</v>
       </c>
-      <c r="I72" s="8" t="n">
+      <c r="I72" s="7" t="n">
         <v>45937.60625</v>
       </c>
       <c r="J72" t="inlineStr">
@@ -12958,13 +12940,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G73" s="8" t="n">
+      <c r="G73" s="7" t="n">
         <v>45915.33055555556</v>
       </c>
-      <c r="H73" s="8" t="n">
+      <c r="H73" s="7" t="n">
         <v>45932.30555555555</v>
       </c>
-      <c r="I73" s="8" t="n">
+      <c r="I73" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J73" t="inlineStr">
@@ -13031,13 +13013,13 @@
           <t>[Ver 2.25]</t>
         </is>
       </c>
-      <c r="G74" s="8" t="n">
+      <c r="G74" s="7" t="n">
         <v>45915.33055555556</v>
       </c>
-      <c r="H74" s="8" t="n">
+      <c r="H74" s="7" t="n">
         <v>45932.60069444445</v>
       </c>
-      <c r="I74" s="8" t="n">
+      <c r="I74" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J74" t="inlineStr">
@@ -13108,13 +13090,13 @@
           <t>[Ver. 2.24.1]</t>
         </is>
       </c>
-      <c r="G75" s="8" t="n">
+      <c r="G75" s="7" t="n">
         <v>45924.79166666666</v>
       </c>
-      <c r="H75" s="8" t="n">
+      <c r="H75" s="7" t="n">
         <v>45926.29861111111</v>
       </c>
-      <c r="I75" s="8" t="n">
+      <c r="I75" s="7" t="n">
         <v>45937.57916666667</v>
       </c>
       <c r="J75" t="inlineStr">
@@ -13189,13 +13171,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G76" s="8" t="n">
+      <c r="G76" s="7" t="n">
         <v>45547.79166666666</v>
       </c>
-      <c r="H76" s="8" t="n">
+      <c r="H76" s="7" t="n">
         <v>45558.79166666666</v>
       </c>
-      <c r="I76" s="8" t="n">
+      <c r="I76" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J76" t="inlineStr">
@@ -13272,13 +13254,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G77" s="8" t="n">
+      <c r="G77" s="7" t="n">
         <v>45545.79166666666</v>
       </c>
-      <c r="H77" s="8" t="n">
+      <c r="H77" s="7" t="n">
         <v>45545.79166666666</v>
       </c>
-      <c r="I77" s="8" t="n">
+      <c r="I77" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J77" t="inlineStr">
@@ -13356,13 +13338,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G78" s="8" t="n">
+      <c r="G78" s="7" t="n">
         <v>45540.79166666666</v>
       </c>
-      <c r="H78" s="8" t="n">
+      <c r="H78" s="7" t="n">
         <v>45543.79166666666</v>
       </c>
-      <c r="I78" s="8" t="n">
+      <c r="I78" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J78" t="inlineStr">
@@ -13440,13 +13422,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G79" s="8" t="n">
+      <c r="G79" s="7" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="H79" s="8" t="n">
+      <c r="H79" s="7" t="n">
         <v>45539.79166666666</v>
       </c>
-      <c r="I79" s="8" t="n">
+      <c r="I79" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J79" t="inlineStr">
@@ -13517,13 +13499,13 @@
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" s="8" t="n">
+      <c r="G80" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="H80" s="8" t="n">
+      <c r="H80" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I80" s="8" t="n">
+      <c r="I80" s="7" t="n">
         <v>45575.79166666666</v>
       </c>
       <c r="J80" t="inlineStr">
@@ -13600,13 +13582,13 @@
           <t>[Ver. 2.18]</t>
         </is>
       </c>
-      <c r="G81" s="8" t="n">
+      <c r="G81" s="7" t="n">
         <v>45559.79166666666</v>
       </c>
-      <c r="H81" s="8" t="n">
+      <c r="H81" s="7" t="n">
         <v>45564.79166666666</v>
       </c>
-      <c r="I81" s="8" t="n">
+      <c r="I81" s="7" t="n">
         <v>45579.79166666666</v>
       </c>
       <c r="J81" t="inlineStr">
@@ -13677,13 +13659,13 @@
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" s="8" t="n">
+      <c r="G82" s="7" t="n">
         <v>45578.79166666666</v>
       </c>
-      <c r="H82" s="8" t="n">
+      <c r="H82" s="7" t="n">
         <v>45585.79166666666</v>
       </c>
-      <c r="I82" s="8" t="n">
+      <c r="I82" s="7" t="n">
         <v>45585.79166666666</v>
       </c>
       <c r="J82" t="inlineStr">
@@ -13754,13 +13736,13 @@
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" s="8" t="n">
+      <c r="G83" s="7" t="n">
         <v>45870.79166666666</v>
       </c>
-      <c r="H83" s="8" t="n">
+      <c r="H83" s="7" t="n">
         <v>45986.79166666666</v>
       </c>
-      <c r="I83" s="8" t="n"/>
+      <c r="I83" s="7" t="n"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>WAPSA Web</t>
@@ -13825,13 +13807,13 @@
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" s="8" t="n">
+      <c r="G84" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="H84" s="8" t="n">
+      <c r="H84" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
-      <c r="I84" s="8" t="n">
+      <c r="I84" s="7" t="n">
         <v>45552.79166666666</v>
       </c>
       <c r="J84" t="inlineStr">
@@ -13902,13 +13884,13 @@
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" s="8" t="n">
+      <c r="G85" s="7" t="n">
         <v>45589.79166666666</v>
       </c>
-      <c r="H85" s="8" t="n">
+      <c r="H85" s="7" t="n">
         <v>45589.79166666666</v>
       </c>
-      <c r="I85" s="8" t="n">
+      <c r="I85" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
       <c r="J85" t="inlineStr">
@@ -13985,13 +13967,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G86" s="8" t="n">
+      <c r="G86" s="7" t="n">
         <v>45592.79166666666</v>
       </c>
-      <c r="H86" s="8" t="n">
+      <c r="H86" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I86" s="8" t="n">
+      <c r="I86" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J86" t="inlineStr">
@@ -14062,13 +14044,13 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" s="8" t="n">
+      <c r="G87" s="7" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H87" s="8" t="n">
+      <c r="H87" s="7" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="I87" s="8" t="n">
+      <c r="I87" s="7" t="n">
         <v>45616.79166666666</v>
       </c>
       <c r="J87" t="inlineStr">
@@ -14141,13 +14123,13 @@
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
-      <c r="G88" s="8" t="n">
+      <c r="G88" s="7" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H88" s="8" t="n">
+      <c r="H88" s="7" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I88" s="8" t="n">
+      <c r="I88" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J88" t="inlineStr">
@@ -14218,13 +14200,13 @@
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" s="8" t="n">
+      <c r="G89" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="H89" s="8" t="n">
+      <c r="H89" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I89" s="8" t="n">
+      <c r="I89" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
       <c r="J89" t="inlineStr">
@@ -14295,13 +14277,13 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" s="8" t="n">
+      <c r="G90" s="7" t="n">
         <v>45595.79166666666</v>
       </c>
-      <c r="H90" s="8" t="n">
+      <c r="H90" s="7" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I90" s="8" t="n">
+      <c r="I90" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J90" t="inlineStr">
@@ -14378,13 +14360,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G91" s="8" t="n">
+      <c r="G91" s="7" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="H91" s="8" t="n">
+      <c r="H91" s="7" t="n">
         <v>45614.79166666666</v>
       </c>
-      <c r="I91" s="8" t="n">
+      <c r="I91" s="7" t="n">
         <v>45662.79166666666</v>
       </c>
       <c r="J91" t="inlineStr">
@@ -14455,13 +14437,13 @@
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
-      <c r="G92" s="8" t="n">
+      <c r="G92" s="7" t="n">
         <v>45608.79166666666</v>
       </c>
-      <c r="H92" s="8" t="n">
+      <c r="H92" s="7" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="I92" s="8" t="n">
+      <c r="I92" s="7" t="n">
         <v>45621.79166666666</v>
       </c>
       <c r="J92" t="inlineStr">
@@ -14538,13 +14520,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G93" s="8" t="n">
+      <c r="G93" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="H93" s="8" t="n">
+      <c r="H93" s="7" t="n">
         <v>45606.79166666666</v>
       </c>
-      <c r="I93" s="8" t="n">
+      <c r="I93" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J93" t="inlineStr">
@@ -14619,13 +14601,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G94" s="8" t="n">
+      <c r="G94" s="7" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="H94" s="8" t="n">
+      <c r="H94" s="7" t="n">
         <v>45617.79166666666</v>
       </c>
-      <c r="I94" s="8" t="n">
+      <c r="I94" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J94" t="inlineStr">
@@ -14700,13 +14682,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G95" s="8" t="n">
+      <c r="G95" s="7" t="n">
         <v>45627.79166666666</v>
       </c>
-      <c r="H95" s="8" t="n">
+      <c r="H95" s="7" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I95" s="8" t="n">
+      <c r="I95" s="7" t="n">
         <v>45671.79166666666</v>
       </c>
       <c r="J95" t="inlineStr">
@@ -14781,13 +14763,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G96" s="8" t="n">
+      <c r="G96" s="7" t="n">
         <v>45623.79166666666</v>
       </c>
-      <c r="H96" s="8" t="n">
+      <c r="H96" s="7" t="n">
         <v>45623.79166666666</v>
       </c>
-      <c r="I96" s="8" t="n">
+      <c r="I96" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J96" t="inlineStr">
@@ -14858,13 +14840,13 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" s="8" t="n">
+      <c r="G97" s="7" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="H97" s="8" t="n">
+      <c r="H97" s="7" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I97" s="8" t="n">
+      <c r="I97" s="7" t="n">
         <v>45680.79166666666</v>
       </c>
       <c r="J97" t="inlineStr">
@@ -14941,13 +14923,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G98" s="8" t="n">
+      <c r="G98" s="7" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="H98" s="8" t="n">
+      <c r="H98" s="7" t="n">
         <v>45389.79166666666</v>
       </c>
-      <c r="I98" s="8" t="n">
+      <c r="I98" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J98" t="inlineStr">
@@ -15018,13 +15000,13 @@
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" s="8" t="n">
+      <c r="G99" s="7" t="n">
         <v>45396.79166666666</v>
       </c>
-      <c r="H99" s="8" t="n">
+      <c r="H99" s="7" t="n">
         <v>45435.79166666666</v>
       </c>
-      <c r="I99" s="8" t="n">
+      <c r="I99" s="7" t="n">
         <v>45435.79166666666</v>
       </c>
       <c r="J99" t="inlineStr">
@@ -15101,13 +15083,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G100" s="8" t="n">
+      <c r="G100" s="7" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="H100" s="8" t="n">
+      <c r="H100" s="7" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="I100" s="8" t="n">
+      <c r="I100" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J100" t="inlineStr">
@@ -15182,13 +15164,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G101" s="8" t="n">
+      <c r="G101" s="7" t="n">
         <v>45398.79166666666</v>
       </c>
-      <c r="H101" s="8" t="n">
+      <c r="H101" s="7" t="n">
         <v>45398.79166666666</v>
       </c>
-      <c r="I101" s="8" t="n">
+      <c r="I101" s="7" t="n">
         <v>45418.79166666666</v>
       </c>
       <c r="J101" t="inlineStr">
@@ -15263,13 +15245,13 @@
           <t>[Ver. 2.16]</t>
         </is>
       </c>
-      <c r="G102" s="8" t="n">
+      <c r="G102" s="7" t="n">
         <v>45424.79166666666</v>
       </c>
-      <c r="H102" s="8" t="n">
+      <c r="H102" s="7" t="n">
         <v>45425.79166666666</v>
       </c>
-      <c r="I102" s="8" t="n">
+      <c r="I102" s="7" t="n">
         <v>45427.79166666666</v>
       </c>
       <c r="J102" t="inlineStr">
@@ -15340,13 +15322,13 @@
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
-      <c r="G103" s="8" t="n">
+      <c r="G103" s="7" t="n">
         <v>45405.79166666666</v>
       </c>
-      <c r="H103" s="8" t="n">
+      <c r="H103" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I103" s="8" t="n">
+      <c r="I103" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
       <c r="J103" t="inlineStr">
@@ -15417,13 +15399,13 @@
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
-      <c r="G104" s="8" t="n">
+      <c r="G104" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="H104" s="8" t="n">
+      <c r="H104" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I104" s="8" t="n">
+      <c r="I104" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
       <c r="J104" t="inlineStr">
@@ -15498,13 +15480,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G105" s="8" t="n">
+      <c r="G105" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="H105" s="8" t="n">
+      <c r="H105" s="7" t="n">
         <v>45432.79166666666</v>
       </c>
-      <c r="I105" s="8" t="n">
+      <c r="I105" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J105" t="inlineStr">
@@ -15579,13 +15561,13 @@
           <t>[2.16.1]</t>
         </is>
       </c>
-      <c r="G106" s="8" t="n">
+      <c r="G106" s="7" t="n">
         <v>45433.79166666666</v>
       </c>
-      <c r="H106" s="8" t="n">
+      <c r="H106" s="7" t="n">
         <v>45433.79166666666</v>
       </c>
-      <c r="I106" s="8" t="n">
+      <c r="I106" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J106" t="inlineStr">
@@ -15656,13 +15638,13 @@
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
-      <c r="G107" s="8" t="n">
+      <c r="G107" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="H107" s="8" t="n">
+      <c r="H107" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
-      <c r="I107" s="8" t="n">
+      <c r="I107" s="7" t="n">
         <v>45438.79166666666</v>
       </c>
       <c r="J107" t="inlineStr">
@@ -15737,13 +15719,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G108" s="8" t="n">
+      <c r="G108" s="7" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="H108" s="8" t="n">
+      <c r="H108" s="7" t="n">
         <v>45342.79166666666</v>
       </c>
-      <c r="I108" s="8" t="n">
+      <c r="I108" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
       <c r="J108" t="inlineStr">
@@ -15820,13 +15802,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G109" s="8" t="n">
+      <c r="G109" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H109" s="8" t="n">
+      <c r="H109" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="I109" s="8" t="n">
+      <c r="I109" s="7" t="n">
         <v>45431.79166666666</v>
       </c>
       <c r="J109" t="inlineStr">
@@ -15901,13 +15883,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G110" s="8" t="n">
+      <c r="G110" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H110" s="8" t="n">
+      <c r="H110" s="7" t="n">
         <v>45361.79166666666</v>
       </c>
-      <c r="I110" s="8" t="n">
+      <c r="I110" s="7" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J110" t="inlineStr">
@@ -15980,13 +15962,13 @@
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
-      <c r="G111" s="8" t="n">
+      <c r="G111" s="7" t="n">
         <v>45368.79166666666</v>
       </c>
-      <c r="H111" s="8" t="n">
+      <c r="H111" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I111" s="8" t="n">
+      <c r="I111" s="7" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J111" t="inlineStr">
@@ -16059,13 +16041,13 @@
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
-      <c r="G112" s="8" t="n">
+      <c r="G112" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="H112" s="8" t="n">
+      <c r="H112" s="7" t="n">
         <v>45369.79166666666</v>
       </c>
-      <c r="I112" s="8" t="n">
+      <c r="I112" s="7" t="n">
         <v>45376.79166666666</v>
       </c>
       <c r="J112" t="inlineStr">
@@ -16136,11 +16118,11 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" s="8" t="n">
+      <c r="G113" s="7" t="n">
         <v>45951.79166666666</v>
       </c>
-      <c r="H113" s="8" t="n"/>
-      <c r="I113" s="8" t="n"/>
+      <c r="H113" s="7" t="n"/>
+      <c r="I113" s="7" t="n"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16205,13 +16187,13 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
-      <c r="G114" s="8" t="n">
+      <c r="G114" s="7" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="H114" s="8" t="n">
+      <c r="H114" s="7" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="I114" s="8" t="n"/>
+      <c r="I114" s="7" t="n"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16284,13 +16266,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G115" s="8" t="n">
+      <c r="G115" s="7" t="n">
         <v>45845.25347222222</v>
       </c>
-      <c r="H115" s="8" t="n">
+      <c r="H115" s="7" t="n">
         <v>45845.79166666666</v>
       </c>
-      <c r="I115" s="8" t="n"/>
+      <c r="I115" s="7" t="n"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16367,13 +16349,13 @@
           <t>[Ver. 4.29]</t>
         </is>
       </c>
-      <c r="G116" s="8" t="n">
+      <c r="G116" s="7" t="n">
         <v>46047.79166666666</v>
       </c>
-      <c r="H116" s="8" t="n">
+      <c r="H116" s="7" t="n">
         <v>46104.26111111111</v>
       </c>
-      <c r="I116" s="8" t="n"/>
+      <c r="I116" s="7" t="n"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16442,13 +16424,13 @@
           <t>[Ver. 2.29]</t>
         </is>
       </c>
-      <c r="G117" s="8" t="n">
+      <c r="G117" s="7" t="n">
         <v>46050.79166666666</v>
       </c>
-      <c r="H117" s="8" t="n">
+      <c r="H117" s="7" t="n">
         <v>46062.46458333333</v>
       </c>
-      <c r="I117" s="8" t="n"/>
+      <c r="I117" s="7" t="n"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16517,13 +16499,13 @@
           <t>[Ver. 2.28]; SLA</t>
         </is>
       </c>
-      <c r="G118" s="8" t="n">
+      <c r="G118" s="7" t="n">
         <v>46090.20833333334</v>
       </c>
-      <c r="H118" s="8" t="n">
+      <c r="H118" s="7" t="n">
         <v>46090.33333333334</v>
       </c>
-      <c r="I118" s="8" t="n"/>
+      <c r="I118" s="7" t="n"/>
       <c r="J118" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -16600,11 +16582,11 @@
           <t>[Ver. 2.28]; SLA</t>
         </is>
       </c>
-      <c r="G119" s="8" t="n">
+      <c r="G119" s="7" t="n">
         <v>46089.79166666666</v>
       </c>
-      <c r="H119" s="8" t="n"/>
-      <c r="I119" s="8" t="n"/>
+      <c r="H119" s="7" t="n"/>
+      <c r="I119" s="7" t="n"/>
       <c r="J119" t="inlineStr">
         <is>
           <t>WapsaWeb</t>
@@ -16669,13 +16651,13 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
-      <c r="G120" s="8" t="n">
+      <c r="G120" s="7" t="n">
         <v>46094.54930555556</v>
       </c>
-      <c r="H120" s="8" t="n">
+      <c r="H120" s="7" t="n">
         <v>46094.54930555556</v>
       </c>
-      <c r="I120" s="8" t="n">
+      <c r="I120" s="7" t="n">
         <v>46097.30972222222</v>
       </c>
       <c r="J120" t="inlineStr">
@@ -16750,13 +16732,13 @@
           <t>[Ver. 2.28]</t>
         </is>
       </c>
-      <c r="G121" s="8" t="n">
+      <c r="G121" s="7" t="n">
         <v>46096.71458333333</v>
       </c>
-      <c r="H121" s="8" t="n">
+      <c r="H121" s="7" t="n">
         <v>46096.71458333333</v>
       </c>
-      <c r="I121" s="8" t="n"/>
+      <c r="I121" s="7" t="n"/>
       <c r="J121" t="inlineStr">
         <is>
           <t>WAPSA</t>
@@ -16825,13 +16807,13 @@
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
-      <c r="G122" s="8" t="n">
+      <c r="G122" s="7" t="n">
         <v>46097.56319444445</v>
       </c>
-      <c r="H122" s="8" t="n">
+      <c r="H122" s="7" t="n">
         <v>46097.56319444445</v>
       </c>
-      <c r="I122" s="8" t="n">
+      <c r="I122" s="7" t="n">
         <v>46097.56319444445</v>
       </c>
       <c r="J122" t="inlineStr">
@@ -16898,9 +16880,9 @@
       </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
-      <c r="G123" s="8" t="n"/>
-      <c r="H123" s="8" t="n"/>
-      <c r="I123" s="8" t="n"/>
+      <c r="G123" s="7" t="n"/>
+      <c r="H123" s="7" t="n"/>
+      <c r="I123" s="7" t="n"/>
       <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="n">
@@ -16953,13 +16935,13 @@
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
-      <c r="G124" s="8" t="n">
+      <c r="G124" s="7" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="H124" s="8" t="n">
+      <c r="H124" s="7" t="n">
         <v>45725.79166666666</v>
       </c>
-      <c r="I124" s="8" t="n">
+      <c r="I124" s="7" t="n">
         <v>45725.79166666666</v>
       </c>
       <c r="J124" t="inlineStr">
@@ -17030,13 +17012,13 @@
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" s="8" t="n">
+      <c r="G125" s="7" t="n">
         <v>45410.79166666666</v>
       </c>
-      <c r="H125" s="8" t="n">
+      <c r="H125" s="7" t="n">
         <v>45454.79166666666</v>
       </c>
-      <c r="I125" s="8" t="n">
+      <c r="I125" s="7" t="n">
         <v>45460.79166666666</v>
       </c>
       <c r="J125" t="inlineStr">
@@ -17109,13 +17091,13 @@
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" s="8" t="n">
+      <c r="G126" s="7" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="H126" s="8" t="n">
+      <c r="H126" s="7" t="n">
         <v>45454.79166666666</v>
       </c>
-      <c r="I126" s="8" t="n">
+      <c r="I126" s="7" t="n">
         <v>45454.79166666666</v>
       </c>
       <c r="J126" t="inlineStr">
@@ -17186,13 +17168,13 @@
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" s="8" t="n">
+      <c r="G127" s="7" t="n">
         <v>45466.79166666666</v>
       </c>
-      <c r="H127" s="8" t="n">
+      <c r="H127" s="7" t="n">
         <v>45466.79166666666</v>
       </c>
-      <c r="I127" s="8" t="n">
+      <c r="I127" s="7" t="n">
         <v>45466.79166666666</v>
       </c>
       <c r="J127" t="inlineStr">
@@ -17263,13 +17245,13 @@
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
-      <c r="G128" s="8" t="n">
+      <c r="G128" s="7" t="n">
         <v>45761.79166666666</v>
       </c>
-      <c r="H128" s="8" t="n">
+      <c r="H128" s="7" t="n">
         <v>45769.79166666666</v>
       </c>
-      <c r="I128" s="8" t="n">
+      <c r="I128" s="7" t="n">
         <v>45809.79166666666</v>
       </c>
       <c r="J128" t="inlineStr">
@@ -17342,13 +17324,13 @@
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
-      <c r="G129" s="8" t="n">
+      <c r="G129" s="7" t="n">
         <v>45747.79166666666</v>
       </c>
-      <c r="H129" s="8" t="n">
+      <c r="H129" s="7" t="n">
         <v>45764.39930555555</v>
       </c>
-      <c r="I129" s="8" t="n">
+      <c r="I129" s="7" t="n">
         <v>45810.79166666666</v>
       </c>
       <c r="J129" t="inlineStr">
@@ -17413,13 +17395,13 @@
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
-      <c r="G130" s="8" t="n">
+      <c r="G130" s="7" t="n">
         <v>45815.29375</v>
       </c>
-      <c r="H130" s="8" t="n">
+      <c r="H130" s="7" t="n">
         <v>45815.37708333333</v>
       </c>
-      <c r="I130" s="8" t="n">
+      <c r="I130" s="7" t="n">
         <v>45822.4375</v>
       </c>
       <c r="J130" t="inlineStr">
@@ -17490,13 +17472,13 @@
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
-      <c r="G131" s="8" t="n">
+      <c r="G131" s="7" t="n">
         <v>45813.79166666666</v>
       </c>
-      <c r="H131" s="8" t="n">
+      <c r="H131" s="7" t="n">
         <v>45818.33819444444</v>
       </c>
-      <c r="I131" s="8" t="n">
+      <c r="I131" s="7" t="n">
         <v>45832.42916666667</v>
       </c>
       <c r="J131" t="inlineStr">
@@ -17567,13 +17549,13 @@
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
-      <c r="G132" s="8" t="n">
+      <c r="G132" s="7" t="n">
         <v>45820.51458333333</v>
       </c>
-      <c r="H132" s="8" t="n">
+      <c r="H132" s="7" t="n">
         <v>45820.51458333333</v>
       </c>
-      <c r="I132" s="8" t="n">
+      <c r="I132" s="7" t="n">
         <v>45827.79166666666</v>
       </c>
       <c r="J132" t="inlineStr">
@@ -17644,13 +17626,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G133" s="8" t="n">
+      <c r="G133" s="7" t="n">
         <v>45851.79166666666</v>
       </c>
-      <c r="H133" s="8" t="n">
+      <c r="H133" s="7" t="n">
         <v>45859.42916666667</v>
       </c>
-      <c r="I133" s="8" t="n"/>
+      <c r="I133" s="7" t="n"/>
       <c r="J133" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -17719,13 +17701,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G134" s="8" t="n">
+      <c r="G134" s="7" t="n">
         <v>45856.60833333333</v>
       </c>
-      <c r="H134" s="8" t="n">
+      <c r="H134" s="7" t="n">
         <v>45856.60833333333</v>
       </c>
-      <c r="I134" s="8" t="n">
+      <c r="I134" s="7" t="n">
         <v>45859.375</v>
       </c>
       <c r="J134" t="inlineStr">
@@ -17796,13 +17778,13 @@
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
-      <c r="G135" s="8" t="n">
+      <c r="G135" s="7" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="H135" s="8" t="n">
+      <c r="H135" s="7" t="n">
         <v>45453.79166666666</v>
       </c>
-      <c r="I135" s="8" t="n">
+      <c r="I135" s="7" t="n">
         <v>45460.79166666666</v>
       </c>
       <c r="J135" t="inlineStr">
@@ -17875,13 +17857,13 @@
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
-      <c r="G136" s="8" t="n">
+      <c r="G136" s="7" t="n">
         <v>45460.79166666666</v>
       </c>
-      <c r="H136" s="8" t="n">
+      <c r="H136" s="7" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="I136" s="8" t="n">
+      <c r="I136" s="7" t="n">
         <v>45490.79166666666</v>
       </c>
       <c r="J136" t="inlineStr">
@@ -17954,13 +17936,13 @@
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
-      <c r="G137" s="8" t="n">
+      <c r="G137" s="7" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="H137" s="8" t="n">
+      <c r="H137" s="7" t="n">
         <v>45461.79166666666</v>
       </c>
-      <c r="I137" s="8" t="n">
+      <c r="I137" s="7" t="n">
         <v>45510.79166666666</v>
       </c>
       <c r="J137" t="inlineStr">
@@ -18033,13 +18015,13 @@
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
-      <c r="G138" s="8" t="n">
+      <c r="G138" s="7" t="n">
         <v>45475.79166666666</v>
       </c>
-      <c r="H138" s="8" t="n">
+      <c r="H138" s="7" t="n">
         <v>45475.79166666666</v>
       </c>
-      <c r="I138" s="8" t="n">
+      <c r="I138" s="7" t="n">
         <v>45475.79166666666</v>
       </c>
       <c r="J138" t="inlineStr">
@@ -18110,13 +18092,13 @@
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="G139" s="8" t="n">
+      <c r="G139" s="7" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="H139" s="8" t="n">
+      <c r="H139" s="7" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="I139" s="8" t="n">
+      <c r="I139" s="7" t="n">
         <v>45479.79166666666</v>
       </c>
       <c r="J139" t="inlineStr">
@@ -18187,13 +18169,13 @@
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" s="8" t="n">
+      <c r="G140" s="7" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="H140" s="8" t="n">
+      <c r="H140" s="7" t="n">
         <v>45487.79166666666</v>
       </c>
-      <c r="I140" s="8" t="n">
+      <c r="I140" s="7" t="n">
         <v>45487.79166666666</v>
       </c>
       <c r="J140" t="inlineStr">
@@ -18264,13 +18246,13 @@
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
-      <c r="G141" s="8" t="n">
+      <c r="G141" s="7" t="n">
         <v>45496.79166666666</v>
       </c>
-      <c r="H141" s="8" t="n">
+      <c r="H141" s="7" t="n">
         <v>45496.79166666666</v>
       </c>
-      <c r="I141" s="8" t="n">
+      <c r="I141" s="7" t="n">
         <v>45496.79166666666</v>
       </c>
       <c r="J141" t="inlineStr">
@@ -18345,13 +18327,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G142" s="8" t="n">
+      <c r="G142" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H142" s="8" t="n">
+      <c r="H142" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I142" s="8" t="n">
+      <c r="I142" s="7" t="n">
         <v>45333.79166666666</v>
       </c>
       <c r="J142" t="inlineStr">
@@ -18426,13 +18408,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G143" s="8" t="n">
+      <c r="G143" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H143" s="8" t="n">
+      <c r="H143" s="7" t="n">
         <v>45334.79166666666</v>
       </c>
-      <c r="I143" s="8" t="n">
+      <c r="I143" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J143" t="inlineStr">
@@ -18507,13 +18489,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G144" s="8" t="n">
+      <c r="G144" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H144" s="8" t="n">
+      <c r="H144" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I144" s="8" t="n">
+      <c r="I144" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J144" t="inlineStr">
@@ -18588,13 +18570,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G145" s="8" t="n">
+      <c r="G145" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H145" s="8" t="n">
+      <c r="H145" s="7" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I145" s="8" t="n">
+      <c r="I145" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J145" t="inlineStr">
@@ -18669,13 +18651,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G146" s="8" t="n">
+      <c r="G146" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H146" s="8" t="n">
+      <c r="H146" s="7" t="n">
         <v>45321.79166666666</v>
       </c>
-      <c r="I146" s="8" t="n">
+      <c r="I146" s="7" t="n">
         <v>45323.79166666666</v>
       </c>
       <c r="J146" t="inlineStr">
@@ -18752,13 +18734,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G147" s="8" t="n">
+      <c r="G147" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H147" s="8" t="n">
+      <c r="H147" s="7" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I147" s="8" t="n">
+      <c r="I147" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J147" t="inlineStr">
@@ -18829,13 +18811,13 @@
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
-      <c r="G148" s="8" t="n">
+      <c r="G148" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H148" s="8" t="n">
+      <c r="H148" s="7" t="n">
         <v>45327.79166666666</v>
       </c>
-      <c r="I148" s="8" t="n">
+      <c r="I148" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J148" t="inlineStr">
@@ -18910,13 +18892,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G149" s="8" t="n">
+      <c r="G149" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H149" s="8" t="n">
+      <c r="H149" s="7" t="n">
         <v>45322.79166666666</v>
       </c>
-      <c r="I149" s="8" t="n">
+      <c r="I149" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J149" t="inlineStr">
@@ -18991,13 +18973,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G150" s="8" t="n">
+      <c r="G150" s="7" t="n">
         <v>45320.79166666666</v>
       </c>
-      <c r="H150" s="8" t="n">
+      <c r="H150" s="7" t="n">
         <v>45321.79166666666</v>
       </c>
-      <c r="I150" s="8" t="n">
+      <c r="I150" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J150" t="inlineStr">
@@ -19072,13 +19054,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G151" s="8" t="n">
+      <c r="G151" s="7" t="n">
         <v>45322.79166666666</v>
       </c>
-      <c r="H151" s="8" t="n">
+      <c r="H151" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I151" s="8" t="n">
+      <c r="I151" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J151" t="inlineStr">
@@ -19155,13 +19137,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G152" s="8" t="n">
+      <c r="G152" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H152" s="8" t="n">
+      <c r="H152" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I152" s="8" t="n">
+      <c r="I152" s="7" t="n">
         <v>45347.79166666666</v>
       </c>
       <c r="J152" t="inlineStr">
@@ -19238,13 +19220,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G153" s="8" t="n">
+      <c r="G153" s="7" t="n">
         <v>45326.79166666666</v>
       </c>
-      <c r="H153" s="8" t="n">
+      <c r="H153" s="7" t="n">
         <v>45326.79166666666</v>
       </c>
-      <c r="I153" s="8" t="n">
+      <c r="I153" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J153" t="inlineStr">
@@ -19325,13 +19307,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G154" s="8" t="n">
+      <c r="G154" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="H154" s="8" t="n">
+      <c r="H154" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="I154" s="8" t="n">
+      <c r="I154" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
       <c r="J154" t="inlineStr">
@@ -19406,13 +19388,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G155" s="8" t="n">
+      <c r="G155" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="H155" s="8" t="n">
+      <c r="H155" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
-      <c r="I155" s="8" t="n">
+      <c r="I155" s="7" t="n">
         <v>45328.79166666666</v>
       </c>
       <c r="J155" t="inlineStr">
@@ -19491,13 +19473,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G156" s="8" t="n">
+      <c r="G156" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="H156" s="8" t="n">
+      <c r="H156" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
-      <c r="I156" s="8" t="n">
+      <c r="I156" s="7" t="n">
         <v>45330.79166666666</v>
       </c>
       <c r="J156" t="inlineStr">
@@ -19568,13 +19550,13 @@
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
-      <c r="G157" s="8" t="n">
+      <c r="G157" s="7" t="n">
         <v>45333.79166666666</v>
       </c>
-      <c r="H157" s="8" t="n">
+      <c r="H157" s="7" t="n">
         <v>45333.79166666666</v>
       </c>
-      <c r="I157" s="8" t="n">
+      <c r="I157" s="7" t="n">
         <v>45340.79166666666</v>
       </c>
       <c r="J157" t="inlineStr">
@@ -19649,13 +19631,13 @@
           <t>Consulta</t>
         </is>
       </c>
-      <c r="G158" s="8" t="n">
+      <c r="G158" s="7" t="n">
         <v>45336.79166666666</v>
       </c>
-      <c r="H158" s="8" t="n">
+      <c r="H158" s="7" t="n">
         <v>45336.79166666666</v>
       </c>
-      <c r="I158" s="8" t="n">
+      <c r="I158" s="7" t="n">
         <v>45336.79166666666</v>
       </c>
       <c r="J158" t="inlineStr">
@@ -19726,13 +19708,13 @@
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
-      <c r="G159" s="8" t="n">
+      <c r="G159" s="7" t="n">
         <v>45347.79166666666</v>
       </c>
-      <c r="H159" s="8" t="n">
+      <c r="H159" s="7" t="n">
         <v>45348.79166666666</v>
       </c>
-      <c r="I159" s="8" t="n">
+      <c r="I159" s="7" t="n">
         <v>45348.79166666666</v>
       </c>
       <c r="J159" t="inlineStr">
@@ -19803,13 +19785,13 @@
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
-      <c r="G160" s="8" t="n">
+      <c r="G160" s="7" t="n">
         <v>46051.25902777778</v>
       </c>
-      <c r="H160" s="8" t="n">
+      <c r="H160" s="7" t="n">
         <v>46051.25902777778</v>
       </c>
-      <c r="I160" s="8" t="n">
+      <c r="I160" s="7" t="n">
         <v>46057.79166666666</v>
       </c>
       <c r="J160" t="inlineStr">
@@ -19876,13 +19858,13 @@
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
-      <c r="G161" s="8" t="n">
+      <c r="G161" s="7" t="n">
         <v>46059.29791666667</v>
       </c>
-      <c r="H161" s="8" t="n">
+      <c r="H161" s="7" t="n">
         <v>46059.29791666667</v>
       </c>
-      <c r="I161" s="8" t="n">
+      <c r="I161" s="7" t="n">
         <v>46062.79166666666</v>
       </c>
       <c r="J161" t="inlineStr">
@@ -19955,13 +19937,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G162" s="8" t="n">
+      <c r="G162" s="7" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="H162" s="8" t="n">
+      <c r="H162" s="7" t="n">
         <v>45670.79166666666</v>
       </c>
-      <c r="I162" s="8" t="n">
+      <c r="I162" s="7" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J162" t="inlineStr">
@@ -20036,13 +20018,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G163" s="8" t="n">
+      <c r="G163" s="7" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="H163" s="8" t="n">
+      <c r="H163" s="7" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="I163" s="8" t="n">
+      <c r="I163" s="7" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J163" t="inlineStr">
@@ -20117,13 +20099,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G164" s="8" t="n">
+      <c r="G164" s="7" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="H164" s="8" t="n">
+      <c r="H164" s="7" t="n">
         <v>45669.79166666666</v>
       </c>
-      <c r="I164" s="8" t="n">
+      <c r="I164" s="7" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J164" t="inlineStr">
@@ -20198,13 +20180,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G165" s="8" t="n">
+      <c r="G165" s="7" t="n">
         <v>45674.79166666666</v>
       </c>
-      <c r="H165" s="8" t="n">
+      <c r="H165" s="7" t="n">
         <v>45674.79166666666</v>
       </c>
-      <c r="I165" s="8" t="n">
+      <c r="I165" s="7" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J165" t="inlineStr">
@@ -20279,13 +20261,13 @@
           <t>[Ver. 2.21]</t>
         </is>
       </c>
-      <c r="G166" s="8" t="n">
+      <c r="G166" s="7" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="H166" s="8" t="n">
+      <c r="H166" s="7" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="I166" s="8" t="n">
+      <c r="I166" s="7" t="n">
         <v>45729.79166666666</v>
       </c>
       <c r="J166" t="inlineStr">
@@ -20360,13 +20342,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G167" s="8" t="n">
+      <c r="G167" s="7" t="n">
         <v>45313.79166666666</v>
       </c>
-      <c r="H167" s="8" t="n">
+      <c r="H167" s="7" t="n">
         <v>45316.79166666666</v>
       </c>
-      <c r="I167" s="8" t="n">
+      <c r="I167" s="7" t="n">
         <v>45316.79166666666</v>
       </c>
       <c r="J167" t="inlineStr">
@@ -20443,13 +20425,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G168" s="8" t="n">
+      <c r="G168" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H168" s="8" t="n">
+      <c r="H168" s="7" t="n">
         <v>45316.79166666666</v>
       </c>
-      <c r="I168" s="8" t="n">
+      <c r="I168" s="7" t="n">
         <v>45319.79166666666</v>
       </c>
       <c r="J168" t="inlineStr">
@@ -20524,13 +20506,13 @@
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
-      <c r="G169" s="8" t="n">
+      <c r="G169" s="7" t="n">
         <v>45986.79166666666</v>
       </c>
-      <c r="H169" s="8" t="n">
+      <c r="H169" s="7" t="n">
         <v>45988.79166666666</v>
       </c>
-      <c r="I169" s="8" t="n">
+      <c r="I169" s="7" t="n">
         <v>46049.79166666666</v>
       </c>
       <c r="J169" t="inlineStr">
@@ -20597,13 +20579,13 @@
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
-      <c r="G170" s="8" t="n">
+      <c r="G170" s="7" t="n">
         <v>46048.33472222222</v>
       </c>
-      <c r="H170" s="8" t="n">
+      <c r="H170" s="7" t="n">
         <v>46048.41805555556</v>
       </c>
-      <c r="I170" s="8" t="n">
+      <c r="I170" s="7" t="n">
         <v>46051.29166666666</v>
       </c>
       <c r="J170" t="inlineStr"/>
@@ -20672,13 +20654,13 @@
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
-      <c r="G171" s="8" t="n">
+      <c r="G171" s="7" t="n">
         <v>45657.79166666666</v>
       </c>
-      <c r="H171" s="8" t="n">
+      <c r="H171" s="7" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="I171" s="8" t="n">
+      <c r="I171" s="7" t="n">
         <v>45662.79166666666</v>
       </c>
       <c r="J171" t="inlineStr">
@@ -20749,13 +20731,13 @@
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
-      <c r="G172" s="8" t="n">
+      <c r="G172" s="7" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="H172" s="8" t="n">
+      <c r="H172" s="7" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="I172" s="8" t="n">
+      <c r="I172" s="7" t="n">
         <v>45683.79166666666</v>
       </c>
       <c r="J172" t="inlineStr">
@@ -20828,13 +20810,13 @@
         </is>
       </c>
       <c r="F173" t="inlineStr"/>
-      <c r="G173" s="8" t="n">
+      <c r="G173" s="7" t="n">
         <v>45662.79166666666</v>
       </c>
-      <c r="H173" s="8" t="n">
+      <c r="H173" s="7" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I173" s="8" t="n">
+      <c r="I173" s="7" t="n">
         <v>45665.79166666666</v>
       </c>
       <c r="J173" t="inlineStr">
@@ -20905,13 +20887,13 @@
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
-      <c r="G174" s="8" t="n">
+      <c r="G174" s="7" t="n">
         <v>45659.79166666666</v>
       </c>
-      <c r="H174" s="8" t="n">
+      <c r="H174" s="7" t="n">
         <v>45663.79166666666</v>
       </c>
-      <c r="I174" s="8" t="n">
+      <c r="I174" s="7" t="n">
         <v>45683.79166666666</v>
       </c>
       <c r="J174" t="inlineStr">
@@ -20978,13 +20960,13 @@
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
-      <c r="G175" s="8" t="n">
+      <c r="G175" s="7" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="H175" s="8" t="n">
+      <c r="H175" s="7" t="n">
         <v>45680.79166666666</v>
       </c>
-      <c r="I175" s="8" t="n">
+      <c r="I175" s="7" t="n">
         <v>45694.79166666666</v>
       </c>
       <c r="J175" t="inlineStr">
@@ -21055,13 +21037,13 @@
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
-      <c r="G176" s="8" t="n">
+      <c r="G176" s="7" t="n">
         <v>45682.79166666666</v>
       </c>
-      <c r="H176" s="8" t="n">
+      <c r="H176" s="7" t="n">
         <v>45683.79166666666</v>
       </c>
-      <c r="I176" s="8" t="n">
+      <c r="I176" s="7" t="n">
         <v>45694.79166666666</v>
       </c>
       <c r="J176" t="inlineStr">
@@ -21134,13 +21116,13 @@
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
-      <c r="G177" s="8" t="n">
+      <c r="G177" s="7" t="n">
         <v>45687.79166666666</v>
       </c>
-      <c r="H177" s="8" t="n">
+      <c r="H177" s="7" t="n">
         <v>45687.79166666666</v>
       </c>
-      <c r="I177" s="8" t="n">
+      <c r="I177" s="7" t="n">
         <v>45688.79166666666</v>
       </c>
       <c r="J177" t="inlineStr">
@@ -21213,13 +21195,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G178" s="8" t="n">
+      <c r="G178" s="7" t="n">
         <v>45963.79166666666</v>
       </c>
-      <c r="H178" s="8" t="n">
+      <c r="H178" s="7" t="n">
         <v>45987.43333333333</v>
       </c>
-      <c r="I178" s="8" t="n"/>
+      <c r="I178" s="7" t="n"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21292,13 +21274,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G179" s="8" t="n">
+      <c r="G179" s="7" t="n">
         <v>45944.79166666666</v>
       </c>
-      <c r="H179" s="8" t="n">
+      <c r="H179" s="7" t="n">
         <v>45951.79166666666</v>
       </c>
-      <c r="I179" s="8" t="n"/>
+      <c r="I179" s="7" t="n"/>
       <c r="J179" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21367,13 +21349,13 @@
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
-      <c r="G180" s="8" t="n">
+      <c r="G180" s="7" t="n">
         <v>45963.79166666666</v>
       </c>
-      <c r="H180" s="8" t="n">
+      <c r="H180" s="7" t="n">
         <v>45979.79166666666</v>
       </c>
-      <c r="I180" s="8" t="n">
+      <c r="I180" s="7" t="n">
         <v>46008.79166666666</v>
       </c>
       <c r="J180" t="inlineStr">
@@ -21444,13 +21426,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G181" s="8" t="n">
+      <c r="G181" s="7" t="n">
         <v>45908.79166666666</v>
       </c>
-      <c r="H181" s="8" t="n">
+      <c r="H181" s="7" t="n">
         <v>45930.79166666666</v>
       </c>
-      <c r="I181" s="8" t="n"/>
+      <c r="I181" s="7" t="n"/>
       <c r="J181" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21519,13 +21501,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G182" s="8" t="n">
+      <c r="G182" s="7" t="n">
         <v>45936.79166666666</v>
       </c>
-      <c r="H182" s="8" t="n">
+      <c r="H182" s="7" t="n">
         <v>45950.79166666666</v>
       </c>
-      <c r="I182" s="8" t="n"/>
+      <c r="I182" s="7" t="n"/>
       <c r="J182" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21590,13 +21572,13 @@
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
-      <c r="G183" s="8" t="n">
+      <c r="G183" s="7" t="n">
         <v>45995.79166666666</v>
       </c>
-      <c r="H183" s="8" t="n">
+      <c r="H183" s="7" t="n">
         <v>46006.29166666666</v>
       </c>
-      <c r="I183" s="8" t="n"/>
+      <c r="I183" s="7" t="n"/>
       <c r="J183" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21665,13 +21647,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G184" s="8" t="n">
+      <c r="G184" s="7" t="n">
         <v>45970.79166666666</v>
       </c>
-      <c r="H184" s="8" t="n">
+      <c r="H184" s="7" t="n">
         <v>45974.51111111111</v>
       </c>
-      <c r="I184" s="8" t="n"/>
+      <c r="I184" s="7" t="n"/>
       <c r="J184" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21740,13 +21722,13 @@
           <t>[Ver 2.26]</t>
         </is>
       </c>
-      <c r="G185" s="8" t="n">
+      <c r="G185" s="7" t="n">
         <v>45981.79166666666</v>
       </c>
-      <c r="H185" s="8" t="n">
+      <c r="H185" s="7" t="n">
         <v>46006.43541666667</v>
       </c>
-      <c r="I185" s="8" t="n"/>
+      <c r="I185" s="7" t="n"/>
       <c r="J185" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -21811,13 +21793,13 @@
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
-      <c r="G186" s="8" t="n">
+      <c r="G186" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="H186" s="8" t="n">
+      <c r="H186" s="7" t="n">
         <v>45628.79166666666</v>
       </c>
-      <c r="I186" s="8" t="n">
+      <c r="I186" s="7" t="n">
         <v>45652.79166666666</v>
       </c>
       <c r="J186" t="inlineStr">
@@ -21890,13 +21872,13 @@
         </is>
       </c>
       <c r="F187" t="inlineStr"/>
-      <c r="G187" s="8" t="n">
+      <c r="G187" s="7" t="n">
         <v>45642.79166666666</v>
       </c>
-      <c r="H187" s="8" t="n">
+      <c r="H187" s="7" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="I187" s="8" t="n">
+      <c r="I187" s="7" t="n">
         <v>45651.79166666666</v>
       </c>
       <c r="J187" t="inlineStr">
@@ -21973,13 +21955,13 @@
           <t>[Ver. 2.19]</t>
         </is>
       </c>
-      <c r="G188" s="8" t="n">
+      <c r="G188" s="7" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="H188" s="8" t="n">
+      <c r="H188" s="7" t="n">
         <v>45652.79166666666</v>
       </c>
-      <c r="I188" s="8" t="n">
+      <c r="I188" s="7" t="n">
         <v>45655.79166666666</v>
       </c>
       <c r="J188" t="inlineStr">
@@ -22054,13 +22036,13 @@
           <t>[Ver 2.24]</t>
         </is>
       </c>
-      <c r="G189" s="8" t="n">
+      <c r="G189" s="7" t="n">
         <v>45820.79166666666</v>
       </c>
-      <c r="H189" s="8" t="n">
+      <c r="H189" s="7" t="n">
         <v>45823.79166666666</v>
       </c>
-      <c r="I189" s="8" t="n"/>
+      <c r="I189" s="7" t="n"/>
       <c r="J189" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -22133,13 +22115,13 @@
           <t>[Ver. 2.17]</t>
         </is>
       </c>
-      <c r="G190" s="8" t="n">
+      <c r="G190" s="7" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="H190" s="8" t="n">
+      <c r="H190" s="7" t="n">
         <v>45481.79166666666</v>
       </c>
-      <c r="I190" s="8" t="n">
+      <c r="I190" s="7" t="n">
         <v>45481.79166666666</v>
       </c>
       <c r="J190" t="inlineStr">
@@ -22210,13 +22192,13 @@
         </is>
       </c>
       <c r="F191" t="inlineStr"/>
-      <c r="G191" s="8" t="n">
+      <c r="G191" s="7" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="H191" s="8" t="n">
+      <c r="H191" s="7" t="n">
         <v>45490.79166666666</v>
       </c>
-      <c r="I191" s="8" t="n">
+      <c r="I191" s="7" t="n">
         <v>45508.79166666666</v>
       </c>
       <c r="J191" t="inlineStr">
@@ -22289,13 +22271,13 @@
         </is>
       </c>
       <c r="F192" t="inlineStr"/>
-      <c r="G192" s="8" t="n">
+      <c r="G192" s="7" t="n">
         <v>45505.79166666666</v>
       </c>
-      <c r="H192" s="8" t="n">
+      <c r="H192" s="7" t="n">
         <v>45505.79166666666</v>
       </c>
-      <c r="I192" s="8" t="n">
+      <c r="I192" s="7" t="n">
         <v>45525.79166666666</v>
       </c>
       <c r="J192" t="inlineStr">
@@ -22368,13 +22350,13 @@
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
-      <c r="G193" s="8" t="n">
+      <c r="G193" s="7" t="n">
         <v>45526.79166666666</v>
       </c>
-      <c r="H193" s="8" t="n">
+      <c r="H193" s="7" t="n">
         <v>45529.79166666666</v>
       </c>
-      <c r="I193" s="8" t="n">
+      <c r="I193" s="7" t="n">
         <v>45529.79166666666</v>
       </c>
       <c r="J193" t="inlineStr">
@@ -22445,13 +22427,13 @@
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
-      <c r="G194" s="8" t="n">
+      <c r="G194" s="7" t="n">
         <v>45528.79166666666</v>
       </c>
-      <c r="H194" s="8" t="n">
+      <c r="H194" s="7" t="n">
         <v>45528.79166666666</v>
       </c>
-      <c r="I194" s="8" t="n">
+      <c r="I194" s="7" t="n">
         <v>45528.79166666666</v>
       </c>
       <c r="J194" t="inlineStr">
@@ -22522,13 +22504,13 @@
         </is>
       </c>
       <c r="F195" t="inlineStr"/>
-      <c r="G195" s="8" t="n">
+      <c r="G195" s="7" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="H195" s="8" t="n">
+      <c r="H195" s="7" t="n">
         <v>45388.79166666666</v>
       </c>
-      <c r="I195" s="8" t="n">
+      <c r="I195" s="7" t="n">
         <v>45397.79166666666</v>
       </c>
       <c r="J195" t="inlineStr">
@@ -22601,13 +22583,13 @@
         </is>
       </c>
       <c r="F196" t="inlineStr"/>
-      <c r="G196" s="8" t="n">
+      <c r="G196" s="7" t="n">
         <v>45392.79166666666</v>
       </c>
-      <c r="H196" s="8" t="n">
+      <c r="H196" s="7" t="n">
         <v>45399.79166666666</v>
       </c>
-      <c r="I196" s="8" t="n">
+      <c r="I196" s="7" t="n">
         <v>45404.79166666666</v>
       </c>
       <c r="J196" t="inlineStr">
@@ -22680,13 +22662,13 @@
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
-      <c r="G197" s="8" t="n">
+      <c r="G197" s="7" t="n">
         <v>45397.79166666666</v>
       </c>
-      <c r="H197" s="8" t="n">
+      <c r="H197" s="7" t="n">
         <v>45397.79166666666</v>
       </c>
-      <c r="I197" s="8" t="n">
+      <c r="I197" s="7" t="n">
         <v>45404.79166666666</v>
       </c>
       <c r="J197" t="inlineStr">
@@ -22759,13 +22741,13 @@
         </is>
       </c>
       <c r="F198" t="inlineStr"/>
-      <c r="G198" s="8" t="n">
+      <c r="G198" s="7" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="H198" s="8" t="n">
+      <c r="H198" s="7" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="I198" s="8" t="n">
+      <c r="I198" s="7" t="n">
         <v>45413.79166666666</v>
       </c>
       <c r="J198" t="inlineStr">
@@ -22836,13 +22818,13 @@
         </is>
       </c>
       <c r="F199" t="inlineStr"/>
-      <c r="G199" s="8" t="n">
+      <c r="G199" s="7" t="n">
         <v>45407.79166666666</v>
       </c>
-      <c r="H199" s="8" t="n">
+      <c r="H199" s="7" t="n">
         <v>45413.79166666666</v>
       </c>
-      <c r="I199" s="8" t="n">
+      <c r="I199" s="7" t="n">
         <v>45413.79166666666</v>
       </c>
       <c r="J199" t="inlineStr">
@@ -22915,13 +22897,13 @@
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
-      <c r="G200" s="8" t="n">
+      <c r="G200" s="7" t="n">
         <v>45693.79166666666</v>
       </c>
-      <c r="H200" s="8" t="n">
+      <c r="H200" s="7" t="n">
         <v>45704.79166666666</v>
       </c>
-      <c r="I200" s="8" t="n">
+      <c r="I200" s="7" t="n">
         <v>45755.44861111111</v>
       </c>
       <c r="J200" t="inlineStr">
@@ -22992,13 +22974,13 @@
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
-      <c r="G201" s="8" t="n">
+      <c r="G201" s="7" t="n">
         <v>45711.79166666666</v>
       </c>
-      <c r="H201" s="8" t="n">
+      <c r="H201" s="7" t="n">
         <v>45712.79166666666</v>
       </c>
-      <c r="I201" s="8" t="n">
+      <c r="I201" s="7" t="n">
         <v>45755.44861111111</v>
       </c>
       <c r="J201" t="inlineStr">
@@ -23073,13 +23055,13 @@
           <t>[Ver. 2.22]</t>
         </is>
       </c>
-      <c r="G202" s="8" t="n">
+      <c r="G202" s="7" t="n">
         <v>45768.79166666666</v>
       </c>
-      <c r="H202" s="8" t="n">
+      <c r="H202" s="7" t="n">
         <v>45770.79166666666</v>
       </c>
-      <c r="I202" s="8" t="n">
+      <c r="I202" s="7" t="n">
         <v>45771.79166666666</v>
       </c>
       <c r="J202" t="inlineStr">
@@ -23150,13 +23132,13 @@
           <t>[Ver.2.14]</t>
         </is>
       </c>
-      <c r="G203" s="8" t="n">
+      <c r="G203" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H203" s="8" t="n">
+      <c r="H203" s="7" t="n">
         <v>45341.79166666666</v>
       </c>
-      <c r="I203" s="8" t="n">
+      <c r="I203" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
       <c r="J203" t="inlineStr">
@@ -23231,13 +23213,13 @@
           <t>[Ver.2.13]</t>
         </is>
       </c>
-      <c r="G204" s="8" t="n">
+      <c r="G204" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="H204" s="8" t="n">
+      <c r="H204" s="7" t="n">
         <v>45314.79166666666</v>
       </c>
-      <c r="I204" s="8" t="n">
+      <c r="I204" s="7" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J204" t="inlineStr">
@@ -23312,13 +23294,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G205" s="8" t="n">
+      <c r="G205" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H205" s="8" t="n">
+      <c r="H205" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I205" s="8" t="n">
+      <c r="I205" s="7" t="n">
         <v>45375.79166666666</v>
       </c>
       <c r="J205" t="inlineStr">
@@ -23393,13 +23375,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G206" s="8" t="n">
+      <c r="G206" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="H206" s="8" t="n">
+      <c r="H206" s="7" t="n">
         <v>45364.79166666666</v>
       </c>
-      <c r="I206" s="8" t="n">
+      <c r="I206" s="7" t="n">
         <v>45375.79166666666</v>
       </c>
       <c r="J206" t="inlineStr">
@@ -23474,13 +23456,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G207" s="8" t="n">
+      <c r="G207" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H207" s="8" t="n">
+      <c r="H207" s="7" t="n">
         <v>45361.79166666666</v>
       </c>
-      <c r="I207" s="8" t="n">
+      <c r="I207" s="7" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J207" t="inlineStr">
@@ -23555,13 +23537,13 @@
           <t>[Ver. 2.15]</t>
         </is>
       </c>
-      <c r="G208" s="8" t="n">
+      <c r="G208" s="7" t="n">
         <v>45355.79166666666</v>
       </c>
-      <c r="H208" s="8" t="n">
+      <c r="H208" s="7" t="n">
         <v>45375.79166666666</v>
       </c>
-      <c r="I208" s="8" t="n">
+      <c r="I208" s="7" t="n">
         <v>45372.79166666666</v>
       </c>
       <c r="J208" t="inlineStr">
@@ -23608,7 +23590,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S208"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A1:S208">
+    <sortState ref="A2:R194">
+      <sortCondition descending="1" ref="C1:C158"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar datos - lun. 01-06-2026
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -7505,7 +7505,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7639,7 +7639,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -10644,7 +10644,7 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -10653,23 +10653,33 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ticket 452 - Guia Remisión Electronica nuevos casos</t>
+          <t>Ticket 453 - Wapsa - Envio datos WAPSA-SAP</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Marzo - 2026</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" s="7" t="n"/>
-      <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>[Ver. 2.25]</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>45930.79166666666</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>45937.45138888889</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>45937.57986111111</v>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10677,12 +10687,16 @@
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="n">
-        <v>452</v>
-      </c>
-      <c r="M44" t="inlineStr"/>
+        <v>453</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/225fb9c5-e533-4606-9111-042ef763c56c?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Mina:&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/63d719b2-06d8-4c83-884f-50e2ce343ba6?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/392f0895-d410-422e-9107-e47dbd4df527?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/d71da09a-4188-4259-a9d4-7cafa283440e?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Callao :&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/20d9850d-70fe-49d7-b2f3-9e2b8b1ba05c?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/f1c8ff88-3eec-49b6-9adc-8d745baf35d4?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Ejecución Manual Envió a SAP:&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/26feb9be-d0fd-4d53-9fc2-39f8c872e02e?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -10711,7 +10725,7 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>486</v>
+        <v>507</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -10720,23 +10734,33 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ticket 454 - Guia Remisión Electronica nuevos casos</t>
+          <t>Ticket 471 - Wapsa - SAP Envio de datos</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Marzo - 2026</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>[Ver. 2.27]; [Ver. 2.28]</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>45991.79166666666</v>
+      </c>
+      <c r="H45" s="7" t="n">
+        <v>46106.79166666666</v>
+      </c>
+      <c r="I45" s="7" t="n">
+        <v>46106.79166666666</v>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10744,12 +10768,16 @@
       </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="n">
-        <v>454</v>
-      </c>
-      <c r="M45" t="inlineStr"/>
+        <v>471</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/27469beb-ea0f-4125-8ece-8774b4e8b960?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/6fd9a9f1-f4d3-41d8-a8b0-630480829703?fileName=image.png" alt=Image style="box-sizing:border-box;max-width:100%;align-self:center;"&gt;&lt;br&gt; &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -10778,7 +10806,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -10787,33 +10815,23 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ticket 453 - Wapsa - Envio datos WAPSA-SAP</t>
+          <t>Ticket 452 - Guia Remisión Electronica nuevos casos</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Marzo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>[Ver. 2.25]</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>45930.79166666666</v>
-      </c>
-      <c r="H46" s="7" t="n">
-        <v>45937.45138888889</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>45937.57986111111</v>
-      </c>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" s="7" t="n"/>
+      <c r="H46" s="7" t="n"/>
+      <c r="I46" s="7" t="n"/>
       <c r="J46" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10821,16 +10839,12 @@
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="n">
-        <v>453</v>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
+        <v>452</v>
+      </c>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Mina:&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/63d719b2-06d8-4c83-884f-50e2ce343ba6?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/392f0895-d410-422e-9107-e47dbd4df527?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/d71da09a-4188-4259-a9d4-7cafa283440e?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Callao :&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/20d9850d-70fe-49d7-b2f3-9e2b8b1ba05c?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/f1c8ff88-3eec-49b6-9adc-8d745baf35d4?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Modulo Ejecución Manual Envió a SAP:&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/26feb9be-d0fd-4d53-9fc2-39f8c872e02e?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/225fb9c5-e533-4606-9111-042ef763c56c?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -10859,7 +10873,7 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>507</v>
+        <v>486</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -10868,33 +10882,23 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ticket 471 - Wapsa - SAP Envio de datos</t>
+          <t>Ticket 454 - Guia Remisión Electronica nuevos casos</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Marzo - 2026</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>[Ver. 2.27]; [Ver. 2.28]</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="n">
-        <v>45991.79166666666</v>
-      </c>
-      <c r="H47" s="7" t="n">
-        <v>46106.79166666666</v>
-      </c>
-      <c r="I47" s="7" t="n">
-        <v>46106.79166666666</v>
-      </c>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" s="7" t="n"/>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -10902,16 +10906,12 @@
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="n">
-        <v>471</v>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
+        <v>454</v>
+      </c>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/6fd9a9f1-f4d3-41d8-a8b0-630480829703?fileName=image.png" alt=Image style="box-sizing:border-box;max-width:100%;align-self:center;"&gt;&lt;br&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/27469beb-ea0f-4125-8ece-8774b4e8b960?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -18781,7 +18781,7 @@
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>377</v>
+        <v>529</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -18790,7 +18790,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Ticket 402 - Wapsa - Callao - E. Shipments - Cuando ocurre un bloqueo al obtener data del Trader Wapsa no muestra el error</t>
+          <t>Ticket 480 - Wapsa - Volteo - Mejora Importacion de pesos</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -18800,15 +18800,19 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="F147" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>[Ver. 2.29]</t>
+        </is>
+      </c>
       <c r="G147" s="7" t="n">
-        <v>45642.79166666666</v>
+        <v>46105.79166666666</v>
       </c>
       <c r="H147" s="7" t="n">
-        <v>45642.79166666666</v>
+        <v>46113.49097222222</v>
       </c>
       <c r="I147" s="7" t="n"/>
       <c r="J147" t="inlineStr">
@@ -18818,18 +18822,14 @@
       </c>
       <c r="K147" t="inlineStr"/>
       <c r="L147" t="n">
-        <v>402</v>
+        <v>480</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
           <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;Cuando se obtienen datos desde el Trader y se genrea algun tipo de error de bloqueo o comunicacion entra ambas Bd's no se muestra: &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/c3f5d344-76e8-4365-9a52-10b27bb70854?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
+      <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -18856,7 +18856,7 @@
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>450</v>
+        <v>535</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -18865,7 +18865,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Ticket 442 - Wapsa - Stock Callao - Error en calculo de TMH en listado detalle por día</t>
+          <t>Ticket 490 - SAP TMS Implementación</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -18875,36 +18875,727 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>[Ver. 2.24]</t>
+          <t>[Ver. 2.29]</t>
         </is>
       </c>
       <c r="G148" s="7" t="n">
-        <v>45845.25347222222</v>
+        <v>46113.46527777778</v>
       </c>
       <c r="H148" s="7" t="n">
-        <v>45845.79166666666</v>
+        <v>46134.79166666666</v>
       </c>
       <c r="I148" s="7" t="n"/>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Wapsa Web</t>
+          <t>WAPSA</t>
         </is>
       </c>
       <c r="K148" t="inlineStr"/>
       <c r="L148" t="n">
+        <v>490</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Requerimiento Nuevo-Area Comercial</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>No implica estabilización</t>
+        </is>
+      </c>
+      <c r="R148" t="n">
+        <v>538</v>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>536</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Ticket 491- Wapsa - Callao - Mejoras Importacion de Leyes</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Mayo - 2026</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>[Ver. 2.29]</t>
+        </is>
+      </c>
+      <c r="G149" s="7" t="n">
+        <v>46120.52361111111</v>
+      </c>
+      <c r="H149" s="7" t="n">
+        <v>46128.79166666666</v>
+      </c>
+      <c r="I149" s="7" t="n"/>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="n">
+        <v>491</v>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Repetitivo-por-resolver</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>A&amp;S</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Estabilización de req. de Mantenimiento</t>
+        </is>
+      </c>
+      <c r="R149" t="n">
+        <v>538</v>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>214</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Ticket 327 - Wapsa - Callao - Ajuste Mensual - Error en Month Evidence historico de Ruma R24-002</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Marzo 2024</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" s="7" t="n">
+        <v>45368.79166666666</v>
+      </c>
+      <c r="H150" s="7" t="n">
+        <v>45369.79166666666</v>
+      </c>
+      <c r="I150" s="7" t="n">
+        <v>45376.79166666666</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>102692</v>
+      </c>
+      <c r="L150" t="n">
+        <v>315</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/6493e66f-26e8-4eb8-a1be-dc375450192d?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;La ruma 45 es parte del historico de la ruma 002 &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;19/03 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp; se envia&amp;nbsp;para firmas de Alejandro &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Repetitivo-en-proceso</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>A&amp;S</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Estabilización de req. de Mantenimiento</t>
+        </is>
+      </c>
+      <c r="R150" t="n">
+        <v>538</v>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>516</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Ticket 474 - Wapsa - Agregar Ajuste D en Reporte de Ajuste Mensual En Linea</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Marzo - 2026</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>[Ver. 2.28]</t>
+        </is>
+      </c>
+      <c r="G151" s="7" t="n">
+        <v>46054.79166666666</v>
+      </c>
+      <c r="H151" s="7" t="n">
+        <v>46062.43472222222</v>
+      </c>
+      <c r="I151" s="7" t="n">
+        <v>46106.79166666666</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="n">
+        <v>474</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Requerimiento Nuevo-Area Comercial</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>No implica estabilización</t>
+        </is>
+      </c>
+      <c r="R151" t="n">
+        <v>538</v>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>527</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Ticket 486 - Wapsa - Ajuste Mensual - Muestra erroneamente los ingresos de la ruma R26-001</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Marzo - 2026</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" s="7" t="n">
+        <v>46097.56319444445</v>
+      </c>
+      <c r="H152" s="7" t="n">
+        <v>46097.56319444445</v>
+      </c>
+      <c r="I152" s="7" t="n">
+        <v>46097.56319444445</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="n">
+        <v>486</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/a6f748b8-2d6a-423d-b875-20010a0b164e?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Solución: &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;El usuario no recordo que no esta contemplado en el lógica moviemientos internos por lo que lo cambio a junta y todo funciono como lo esperado &lt;/div&gt;&lt;div&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Error del usuario</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>No implica estabilización</t>
+        </is>
+      </c>
+      <c r="R152" t="n">
+        <v>538</v>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>362</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Ticket 397 - Wapsa - Callao - Evidence Of Shipments - Evidence of Shipment nuevo caso NC</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Marzo - 2025</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" s="7" t="n">
+        <v>45725.79166666666</v>
+      </c>
+      <c r="H153" s="7" t="n">
+        <v>45725.79166666666</v>
+      </c>
+      <c r="I153" s="7" t="n">
+        <v>45725.79166666666</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="n">
+        <v>397</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Se requiere considerar nuevo caso que viene de la vista del Trader para ser consumido por el modulo del wapsa Evidence of shipment.&amp;nbsp; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Nicolas se hará cargo de la modificación &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Luego tenemos que importar y ver esta operación &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Solución:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>A&amp;S</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Estabilización de req. de Mantenimiento</t>
+        </is>
+      </c>
+      <c r="R153" t="n">
+        <v>538</v>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>234</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Ticket 344 - Wapsa - Callao - Lista Despacho - Alerta despachos pesos 0 no manda datos sobre las IE's</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Junio 2024</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" s="7" t="n">
+        <v>45410.79166666666</v>
+      </c>
+      <c r="H154" s="7" t="n">
+        <v>45454.79166666666</v>
+      </c>
+      <c r="I154" s="7" t="n">
+        <v>45460.79166666666</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>109586</v>
+      </c>
+      <c r="L154" t="n">
+        <v>344</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/83c9d948-689e-4ab1-88be-3336f3a5a233?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;a href="#" data-vss-mention="version:2.0,758aadd7-85a1-6893-9bad-8face9b229c8"&gt;@Frank Macavilca&lt;/a&gt;&amp;nbsp;la IE en cuestion no ha cumplido los 7 dias de registrada hasta la fecha y pos eso no sale en el listado &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/12b0b23a-f9f8-4862-ba1c-6120f6c4bdf5?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;04/06&amp;nbsp;&lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se corrige listado para que filtre correctamnete utilizando los lotes actual y el anterior. &lt;/div&gt;&lt;div&gt;Se enviara como tikcet. Se envia un formato para firma de AM &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;AM Envia docuemento firmado. Se adjunta &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Wally solicita en reunion del 11/06, que el listado incluya un lote mas hacia atras del tiempo. Se haran los cambios. S emueve Ticket a estado en Desarrollo &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se agrega cambio al script y se envia a TICA 12/06/2023 13:24 pm &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Repetitivo-en-proceso</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>A&amp;S</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Estabilización de req. de Mantenimiento</t>
+        </is>
+      </c>
+      <c r="R154" t="n">
+        <v>538</v>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>268</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Ticket 361 - Wapsa - Callao - Ajuste Mensual - Problema en  ajuste en línea R24-013 - JUNIO</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Junio 2024</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" s="7" t="n">
+        <v>45466.79166666666</v>
+      </c>
+      <c r="H155" s="7" t="n">
+        <v>45466.79166666666</v>
+      </c>
+      <c r="I155" s="7" t="n">
+        <v>45466.79166666666</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="n">
+        <v>361</v>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;Diego Cardenas reporta&amp;nbsp; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/b7318f47-b451-4aa8-b5d8-729247a0d339?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;24/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se detecta un repeso total duplicado: &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/0b3e7192-c054-4a41-a921-7f64bd67bee5?fileName=WhatsApp%20Image%202024-06-24%20at%2016.49.35.jpeg" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;a href="#" data-vss-mention="version:2.0,758aadd7-85a1-6893-9bad-8face9b229c8"&gt;@Frank Macavilca&lt;/a&gt;&amp;nbsp;&amp;nbsp;Responde via mail &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/51ef8424-2061-4f19-9ade-d42b9a5351cf?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>Error del usuario</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>No implica estabilización</t>
+        </is>
+      </c>
+      <c r="R155" t="n">
+        <v>538</v>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>377</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Ticket 402 - Wapsa - Callao - E. Shipments - Cuando ocurre un bloqueo al obtener data del Trader Wapsa no muestra el error</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Junio - 2026</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" s="7" t="n">
+        <v>45642.79166666666</v>
+      </c>
+      <c r="H156" s="7" t="n">
+        <v>45642.79166666666</v>
+      </c>
+      <c r="I156" s="7" t="n"/>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="n">
+        <v>402</v>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;Cuando se obtienen datos desde el Trader y se genrea algun tipo de error de bloqueo o comunicacion entra ambas Bd's no se muestra: &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/c3f5d344-76e8-4365-9a52-10b27bb70854?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>A&amp;S</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Estabilización de req. de Mantenimiento</t>
+        </is>
+      </c>
+      <c r="R156" t="n">
+        <v>538</v>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>Callao</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>450</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Ticket</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Ticket 442 - Wapsa - Stock Callao - Error en calculo de TMH en listado detalle por día</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>WAPSA\Sprint - Junio - 2026</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>[Ver. 2.24]</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="n">
+        <v>45845.25347222222</v>
+      </c>
+      <c r="H157" s="7" t="n">
+        <v>45845.79166666666</v>
+      </c>
+      <c r="I157" s="7" t="n"/>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Wapsa Web</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="n">
         <v>442</v>
       </c>
-      <c r="M148" t="inlineStr">
+      <c r="M157" t="inlineStr">
         <is>
           <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N148" t="inlineStr">
+      <c r="N157" t="inlineStr">
         <is>
           <t>&lt;div&gt;&lt;p style="margin:0cm;font-size:11pt;font-family:Calibri, sans-serif;"&gt;Este ticket tiene como objetivo atender el requerimiento de
 Diego Cárdenas el cual ha detecto que se debe cambiar la fecha que utiliza el
@@ -18913,681 +19604,14 @@
 la de otros reportes. &lt;/p&gt;&lt;br&gt; &lt;/div&gt;</t>
         </is>
       </c>
-      <c r="O148" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P148" t="inlineStr">
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
         <is>
           <t>S&amp;C Sistemas</t>
-        </is>
-      </c>
-      <c r="Q148" t="inlineStr">
-        <is>
-          <t>Estabilización de req. de Mantenimiento</t>
-        </is>
-      </c>
-      <c r="R148" t="n">
-        <v>538</v>
-      </c>
-      <c r="S148" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="n">
-        <v>529</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Ticket 480 - Wapsa - Volteo - Mejora Importacion de pesos</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>[Ver. 2.29]</t>
-        </is>
-      </c>
-      <c r="G149" s="7" t="n">
-        <v>46105.79166666666</v>
-      </c>
-      <c r="H149" s="7" t="n">
-        <v>46113.49097222222</v>
-      </c>
-      <c r="I149" s="7" t="n"/>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="n">
-        <v>480</v>
-      </c>
-      <c r="M149" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P149" t="inlineStr">
-        <is>
-          <t>A&amp;S</t>
-        </is>
-      </c>
-      <c r="Q149" t="inlineStr">
-        <is>
-          <t>Estabilización de req. de Mantenimiento</t>
-        </is>
-      </c>
-      <c r="R149" t="n">
-        <v>538</v>
-      </c>
-      <c r="S149" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>535</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Ticket 490 - SAP TMS Implementación</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>[Ver. 2.29]</t>
-        </is>
-      </c>
-      <c r="G150" s="7" t="n">
-        <v>46113.46527777778</v>
-      </c>
-      <c r="H150" s="7" t="n">
-        <v>46134.79166666666</v>
-      </c>
-      <c r="I150" s="7" t="n"/>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>WAPSA</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr"/>
-      <c r="L150" t="n">
-        <v>490</v>
-      </c>
-      <c r="M150" t="inlineStr">
-        <is>
-          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P150" t="inlineStr">
-        <is>
-          <t>Requerimiento Nuevo-Area Comercial</t>
-        </is>
-      </c>
-      <c r="Q150" t="inlineStr">
-        <is>
-          <t>No implica estabilización</t>
-        </is>
-      </c>
-      <c r="R150" t="n">
-        <v>538</v>
-      </c>
-      <c r="S150" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>536</v>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Ticket 491- Wapsa - Callao - Mejoras Importacion de Leyes</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Resuelto</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>[Ver. 2.29]</t>
-        </is>
-      </c>
-      <c r="G151" s="7" t="n">
-        <v>46120.52361111111</v>
-      </c>
-      <c r="H151" s="7" t="n">
-        <v>46128.79166666666</v>
-      </c>
-      <c r="I151" s="7" t="n"/>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr"/>
-      <c r="L151" t="n">
-        <v>491</v>
-      </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr">
-        <is>
-          <t>Repetitivo-por-resolver</t>
-        </is>
-      </c>
-      <c r="P151" t="inlineStr">
-        <is>
-          <t>A&amp;S</t>
-        </is>
-      </c>
-      <c r="Q151" t="inlineStr">
-        <is>
-          <t>Estabilización de req. de Mantenimiento</t>
-        </is>
-      </c>
-      <c r="R151" t="n">
-        <v>538</v>
-      </c>
-      <c r="S151" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="n">
-        <v>542</v>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Ticket 493 - Wapsa - Callao - Utilizar Fechamcp para las operaciones de ingresos</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
-        </is>
-      </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" s="7" t="n"/>
-      <c r="H152" s="7" t="n"/>
-      <c r="I152" s="7" t="n"/>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
-      <c r="M152" t="inlineStr"/>
-      <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P152" t="inlineStr"/>
-      <c r="Q152" t="inlineStr"/>
-      <c r="R152" t="n">
-        <v>538</v>
-      </c>
-      <c r="S152" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="n">
-        <v>214</v>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Ticket 327 - Wapsa - Callao - Ajuste Mensual - Error en Month Evidence historico de Ruma R24-002</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Marzo 2024</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" s="7" t="n">
-        <v>45368.79166666666</v>
-      </c>
-      <c r="H153" s="7" t="n">
-        <v>45369.79166666666</v>
-      </c>
-      <c r="I153" s="7" t="n">
-        <v>45376.79166666666</v>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K153" t="n">
-        <v>102692</v>
-      </c>
-      <c r="L153" t="n">
-        <v>315</v>
-      </c>
-      <c r="M153" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N153" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/6493e66f-26e8-4eb8-a1be-dc375450192d?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;La ruma 45 es parte del historico de la ruma 002 &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;19/03 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp; se envia&amp;nbsp;para firmas de Alejandro &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="O153" t="inlineStr">
-        <is>
-          <t>Repetitivo-en-proceso</t>
-        </is>
-      </c>
-      <c r="P153" t="inlineStr">
-        <is>
-          <t>A&amp;S</t>
-        </is>
-      </c>
-      <c r="Q153" t="inlineStr">
-        <is>
-          <t>Estabilización de req. de Mantenimiento</t>
-        </is>
-      </c>
-      <c r="R153" t="n">
-        <v>538</v>
-      </c>
-      <c r="S153" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="n">
-        <v>516</v>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Ticket 474 - Wapsa - Agregar Ajuste D en Reporte de Ajuste Mensual En Linea</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Marzo - 2026</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>[Ver. 2.28]</t>
-        </is>
-      </c>
-      <c r="G154" s="7" t="n">
-        <v>46054.79166666666</v>
-      </c>
-      <c r="H154" s="7" t="n">
-        <v>46062.43472222222</v>
-      </c>
-      <c r="I154" s="7" t="n">
-        <v>46106.79166666666</v>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K154" t="inlineStr"/>
-      <c r="L154" t="n">
-        <v>474</v>
-      </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N154" t="inlineStr"/>
-      <c r="O154" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P154" t="inlineStr">
-        <is>
-          <t>Requerimiento Nuevo-Area Comercial</t>
-        </is>
-      </c>
-      <c r="Q154" t="inlineStr">
-        <is>
-          <t>No implica estabilización</t>
-        </is>
-      </c>
-      <c r="R154" t="n">
-        <v>538</v>
-      </c>
-      <c r="S154" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="n">
-        <v>527</v>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Ticket 486 - Wapsa - Ajuste Mensual - Muestra erroneamente los ingresos de la ruma R26-001</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Marzo - 2026</t>
-        </is>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" s="7" t="n">
-        <v>46097.56319444445</v>
-      </c>
-      <c r="H155" s="7" t="n">
-        <v>46097.56319444445</v>
-      </c>
-      <c r="I155" s="7" t="n">
-        <v>46097.56319444445</v>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr"/>
-      <c r="L155" t="n">
-        <v>486</v>
-      </c>
-      <c r="M155" t="inlineStr">
-        <is>
-          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N155" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/a6f748b8-2d6a-423d-b875-20010a0b164e?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Solución: &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;El usuario no recordo que no esta contemplado en el lógica moviemientos internos por lo que lo cambio a junta y todo funciono como lo esperado &lt;/div&gt;&lt;div&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="O155" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P155" t="inlineStr">
-        <is>
-          <t>Error del usuario</t>
-        </is>
-      </c>
-      <c r="Q155" t="inlineStr">
-        <is>
-          <t>No implica estabilización</t>
-        </is>
-      </c>
-      <c r="R155" t="n">
-        <v>538</v>
-      </c>
-      <c r="S155" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="n">
-        <v>362</v>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Ticket 397 - Wapsa - Callao - Evidence Of Shipments - Evidence of Shipment nuevo caso NC</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Marzo - 2025</t>
-        </is>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" s="7" t="n">
-        <v>45725.79166666666</v>
-      </c>
-      <c r="H156" s="7" t="n">
-        <v>45725.79166666666</v>
-      </c>
-      <c r="I156" s="7" t="n">
-        <v>45725.79166666666</v>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="n">
-        <v>397</v>
-      </c>
-      <c r="M156" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N156" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Se requiere considerar nuevo caso que viene de la vista del Trader para ser consumido por el modulo del wapsa Evidence of shipment.&amp;nbsp; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Nicolas se hará cargo de la modificación &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Luego tenemos que importar y ver esta operación &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Solución:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="O156" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="P156" t="inlineStr">
-        <is>
-          <t>A&amp;S</t>
-        </is>
-      </c>
-      <c r="Q156" t="inlineStr">
-        <is>
-          <t>Estabilización de req. de Mantenimiento</t>
-        </is>
-      </c>
-      <c r="R156" t="n">
-        <v>538</v>
-      </c>
-      <c r="S156" t="inlineStr">
-        <is>
-          <t>Callao</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="n">
-        <v>234</v>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Ticket</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Ticket 344 - Wapsa - Callao - Lista Despacho - Alerta despachos pesos 0 no manda datos sobre las IE's</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>WAPSA\Sprint - Junio 2024</t>
-        </is>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Cerrado</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" s="7" t="n">
-        <v>45410.79166666666</v>
-      </c>
-      <c r="H157" s="7" t="n">
-        <v>45454.79166666666</v>
-      </c>
-      <c r="I157" s="7" t="n">
-        <v>45460.79166666666</v>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>Wapsa Web</t>
-        </is>
-      </c>
-      <c r="K157" t="n">
-        <v>109586</v>
-      </c>
-      <c r="L157" t="n">
-        <v>344</v>
-      </c>
-      <c r="M157" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N157" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/83c9d948-689e-4ab1-88be-3336f3a5a233?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;a href="#" data-vss-mention="version:2.0,758aadd7-85a1-6893-9bad-8face9b229c8"&gt;@Frank Macavilca&lt;/a&gt;&amp;nbsp;la IE en cuestion no ha cumplido los 7 dias de registrada hasta la fecha y pos eso no sale en el listado &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/12b0b23a-f9f8-4862-ba1c-6120f6c4bdf5?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;04/06&amp;nbsp;&lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se corrige listado para que filtre correctamnete utilizando los lotes actual y el anterior. &lt;/div&gt;&lt;div&gt;Se enviara como tikcet. Se envia un formato para firma de AM &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;AM Envia docuemento firmado. Se adjunta &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Wally solicita en reunion del 11/06, que el listado incluya un lote mas hacia atras del tiempo. Se haran los cambios. S emueve Ticket a estado en Desarrollo &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se agrega cambio al script y se envia a TICA 12/06/2023 13:24 pm &lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="O157" t="inlineStr">
-        <is>
-          <t>Repetitivo-en-proceso</t>
-        </is>
-      </c>
-      <c r="P157" t="inlineStr">
-        <is>
-          <t>A&amp;S</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr">
@@ -19606,7 +19630,7 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>268</v>
+        <v>542</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -19615,29 +19639,25 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Ticket 361 - Wapsa - Callao - Ajuste Mensual - Problema en  ajuste en línea R24-013 - JUNIO</t>
+          <t>Ticket 493 - Wapsa - Callao - Utilizar Fechamcp para las operaciones de ingresos</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Junio 2024</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Cerrado</t>
+          <t>En Testing</t>
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
       <c r="G158" s="7" t="n">
-        <v>45466.79166666666</v>
-      </c>
-      <c r="H158" s="7" t="n">
-        <v>45466.79166666666</v>
-      </c>
-      <c r="I158" s="7" t="n">
-        <v>45466.79166666666</v>
-      </c>
+        <v>46155.79166666666</v>
+      </c>
+      <c r="H158" s="7" t="n"/>
+      <c r="I158" s="7" t="n"/>
       <c r="J158" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -19645,18 +19665,14 @@
       </c>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="n">
-        <v>361</v>
+        <v>493</v>
       </c>
       <c r="M158" t="inlineStr">
         <is>
           <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;Diego Cardenas reporta&amp;nbsp; &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/b7318f47-b451-4aa8-b5d8-729247a0d339?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;24/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Se detecta un repeso total duplicado: &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/0b3e7192-c054-4a41-a921-7f64bd67bee5?fileName=WhatsApp%20Image%202024-06-24%20at%2016.49.35.jpeg" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;a href="#" data-vss-mention="version:2.0,758aadd7-85a1-6893-9bad-8face9b229c8"&gt;@Frank Macavilca&lt;/a&gt;&amp;nbsp;&amp;nbsp;Responde via mail &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/51ef8424-2061-4f19-9ade-d42b9a5351cf?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
+      <c r="N158" t="inlineStr"/>
       <c r="O158" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -19664,12 +19680,12 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>Error del usuario</t>
+          <t>Requerimiento Nuevo-Area Comercial</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>No implica estabilización</t>
+          <t>Estabilización de req. de Mantenimiento</t>
         </is>
       </c>
       <c r="R158" t="n">
@@ -23360,7 +23376,7 @@
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>340</v>
+        <v>518</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -23369,7 +23385,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Ticket 384 - Wapsa - General - Configuracion -  Crear Modulo para guardar las plantilla de importacion de datos</t>
+          <t>Ticket 476 - Wapsa -Varios - Mejora Listado para elegir vagones en Arribo, Entrega y Salida</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -23379,14 +23395,20 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
-      <c r="F206" t="inlineStr"/>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>[Ver. 2.29]</t>
+        </is>
+      </c>
       <c r="G206" s="7" t="n">
-        <v>45951.79166666666</v>
-      </c>
-      <c r="H206" s="7" t="n"/>
+        <v>46047.79166666666</v>
+      </c>
+      <c r="H206" s="7" t="n">
+        <v>46104.26111111111</v>
+      </c>
       <c r="I206" s="7" t="n"/>
       <c r="J206" t="inlineStr">
         <is>
@@ -23395,14 +23417,14 @@
       </c>
       <c r="K206" t="inlineStr"/>
       <c r="L206" t="n">
-        <v>384</v>
-      </c>
-      <c r="M206" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N206" t="inlineStr"/>
+        <v>476</v>
+      </c>
+      <c r="M206" t="inlineStr"/>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/8562dbaa-6874-4c02-b55e-12a8ad13591f?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
       <c r="O206" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23429,7 +23451,7 @@
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -23438,7 +23460,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Ticket 476 - Wapsa -Varios - Mejora Listado para elegir vagones en Arribo, Entrega y Salida</t>
+          <t>Ticket 486 - Wapsa - Lotes - Validar que la hora de cierre del lote sea únicamente 06:59</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -23448,7 +23470,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Resuelto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
@@ -23457,10 +23479,10 @@
         </is>
       </c>
       <c r="G207" s="7" t="n">
-        <v>46047.79166666666</v>
+        <v>46050.79166666666</v>
       </c>
       <c r="H207" s="7" t="n">
-        <v>46104.26111111111</v>
+        <v>46062.46458333333</v>
       </c>
       <c r="I207" s="7" t="n"/>
       <c r="J207" t="inlineStr">
@@ -23470,14 +23492,14 @@
       </c>
       <c r="K207" t="inlineStr"/>
       <c r="L207" t="n">
-        <v>476</v>
-      </c>
-      <c r="M207" t="inlineStr"/>
-      <c r="N207" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/8562dbaa-6874-4c02-b55e-12a8ad13591f?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
+        <v>486</v>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr"/>
       <c r="O207" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23504,7 +23526,7 @@
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -23513,7 +23535,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Ticket 486 - Wapsa - Lotes - Validar que la hora de cierre del lote sea únicamente 06:59</t>
+          <t>Ticket 482 - Wapsa - Lista de Despacho - No muestra la informacion del campo Almacen vacíos al ver la IE</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -23523,19 +23545,19 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Resuelto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>[Ver. 2.29]</t>
+          <t>[Ver. 2.29]; SLA</t>
         </is>
       </c>
       <c r="G208" s="7" t="n">
-        <v>46050.79166666666</v>
+        <v>46090.20833333334</v>
       </c>
       <c r="H208" s="7" t="n">
-        <v>46062.46458333333</v>
+        <v>46090.33333333334</v>
       </c>
       <c r="I208" s="7" t="n"/>
       <c r="J208" t="inlineStr">
@@ -23543,16 +23565,24 @@
           <t>Wapsa Web</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>SLA</t>
+        </is>
+      </c>
       <c r="L208" t="n">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
           <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N208" t="inlineStr"/>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/0caa4914-6dfb-43dc-acba-dc8d7e950b43?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Corregido siguiente pase &lt;/div&gt;&lt;div&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
       <c r="O208" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23560,7 +23590,7 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>S&amp;C Sistemas</t>
+          <t>A&amp;S</t>
         </is>
       </c>
       <c r="Q208" t="inlineStr">
@@ -23579,7 +23609,7 @@
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -23588,7 +23618,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Ticket 482 - Wapsa - Lista de Despacho - No muestra la informacion del campo Almacen vacíos al ver la IE</t>
+          <t>Ticket 492-  Wapsa - Incrementar tiempo de sesion del usuario MCP</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -23598,19 +23628,19 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Resuelto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>[Ver. 2.29]; SLA</t>
+          <t>[Ver. 2.29]</t>
         </is>
       </c>
       <c r="G209" s="7" t="n">
-        <v>46090.20833333334</v>
+        <v>46128.79166666666</v>
       </c>
       <c r="H209" s="7" t="n">
-        <v>46090.33333333334</v>
+        <v>46129.80625</v>
       </c>
       <c r="I209" s="7" t="n"/>
       <c r="J209" t="inlineStr">
@@ -23618,24 +23648,16 @@
           <t>Wapsa Web</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>SLA</t>
-        </is>
-      </c>
+      <c r="K209" t="inlineStr"/>
       <c r="L209" t="n">
-        <v>482</v>
+        <v>492</v>
       </c>
       <c r="M209" t="inlineStr">
         <is>
           <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N209" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/0caa4914-6dfb-43dc-acba-dc8d7e950b43?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;Corregido siguiente pase &lt;/div&gt;&lt;div&gt; &lt;/div&gt;</t>
-        </is>
-      </c>
+      <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23643,7 +23665,7 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>A&amp;S</t>
+          <t>Requerimiento Nuevo-Area Comercial</t>
         </is>
       </c>
       <c r="Q209" t="inlineStr">
@@ -23662,7 +23684,7 @@
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>541</v>
+        <v>524</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -23671,31 +23693,33 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Ticket 492-  Wapsa - Incrementar tiempo de sesion del usuario MCP</t>
+          <t>Ticket 483 - Wapsa - Lista de Despacho - Error de formato de fechas al exportar detalle de despachos de pesos de una IE</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Mayo - 2026</t>
+          <t>WAPSA\Sprint - Marzo - 2026</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Resuelto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>[Ver. 2.29]</t>
+          <t>[Ver. 2.28]; SLA</t>
         </is>
       </c>
       <c r="G210" s="7" t="n">
-        <v>46128.79166666666</v>
+        <v>46089.79166666666</v>
       </c>
       <c r="H210" s="7" t="n">
-        <v>46129.80625</v>
-      </c>
-      <c r="I210" s="7" t="n"/>
+        <v>46089.79166666666</v>
+      </c>
+      <c r="I210" s="7" t="n">
+        <v>46089.79166666666</v>
+      </c>
       <c r="J210" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -23703,14 +23727,14 @@
       </c>
       <c r="K210" t="inlineStr"/>
       <c r="L210" t="n">
-        <v>492</v>
-      </c>
-      <c r="M210" t="inlineStr">
-        <is>
-          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
-        </is>
-      </c>
-      <c r="N210" t="inlineStr"/>
+        <v>483</v>
+      </c>
+      <c r="M210" t="inlineStr"/>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>&lt;div&gt;Al importar información como Guías/Pesos a una IE de la Lista de Despacho el formato de fecha esta errado, WAPSA interpreta erróneamente la info y graba la fecha con un formato distinto al del Excel de importación, favor corregir ya que no esta quedando grabada correctamente la información en WAPSA.&lt;br&gt; &lt;/div&gt;</t>
+        </is>
+      </c>
       <c r="O210" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23718,7 +23742,7 @@
       </c>
       <c r="P210" t="inlineStr">
         <is>
-          <t>Requerimiento Nuevo-Area Comercial</t>
+          <t>Omisión del usuario</t>
         </is>
       </c>
       <c r="Q210" t="inlineStr">
@@ -23737,7 +23761,7 @@
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -23746,7 +23770,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Ticket 483 - Wapsa - Lista de Despacho - Error de formato de fechas al exportar detalle de despachos de pesos de una IE</t>
+          <t>Ticket 485 - WAPSA - Ajuste Final no deja registrar debido a validacion</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -23761,31 +23785,33 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>[Ver. 2.28]; SLA</t>
+          <t>[Ver. 2.28]</t>
         </is>
       </c>
       <c r="G211" s="7" t="n">
-        <v>46089.79166666666</v>
+        <v>46096.71458333333</v>
       </c>
       <c r="H211" s="7" t="n">
-        <v>46089.79166666666</v>
-      </c>
-      <c r="I211" s="7" t="n">
-        <v>46089.79166666666</v>
-      </c>
+        <v>46096.71458333333</v>
+      </c>
+      <c r="I211" s="7" t="n"/>
       <c r="J211" t="inlineStr">
         <is>
-          <t>Wapsa Web</t>
+          <t>WAPSA</t>
         </is>
       </c>
       <c r="K211" t="inlineStr"/>
       <c r="L211" t="n">
-        <v>483</v>
-      </c>
-      <c r="M211" t="inlineStr"/>
+        <v>485</v>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+        </is>
+      </c>
       <c r="N211" t="inlineStr">
         <is>
-          <t>&lt;div&gt;Al importar información como Guías/Pesos a una IE de la Lista de Despacho el formato de fecha esta errado, WAPSA interpreta erróneamente la info y graba la fecha con un formato distinto al del Excel de importación, favor corregir ya que no esta quedando grabada correctamente la información en WAPSA.&lt;br&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;He registrado el ultimo movimiento de esa ruma a las 23:00 hrs del 14/03, el ajuste lo estoy poniendo como 14/03 23:59, por que si le pongo 15/03 que fue en realidad la operación me sale otro error que dice que la fecha no puede ser posterior a la fecha de resumen&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/9970cbf3-cd07-41b8-8c16-d3ff09d6b2f6?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Solución:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O211" t="inlineStr">
@@ -23795,12 +23821,12 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>Omisión del usuario</t>
+          <t>S&amp;C Sistemas</t>
         </is>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
-          <t>No implica estabilización</t>
+          <t>Estabilización por proyecto</t>
         </is>
       </c>
       <c r="R211" t="n">
@@ -23814,7 +23840,7 @@
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>526</v>
+        <v>255</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -23823,12 +23849,12 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Ticket 485 - WAPSA - Ajuste Final no deja registrar debido a validacion</t>
+          <t>Ticket 358 - Wapsa - General - Informacion sobre propuesta de mejoras para los Pases a produccion, tickets y ambientes de pruebas</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Marzo - 2026</t>
+          <t>WAPSA\Sprint - Junio 2024</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -23836,35 +23862,33 @@
           <t>Cerrado</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr">
-        <is>
-          <t>[Ver. 2.28]</t>
-        </is>
-      </c>
+      <c r="F212" t="inlineStr"/>
       <c r="G212" s="7" t="n">
-        <v>46096.71458333333</v>
+        <v>45453.79166666666</v>
       </c>
       <c r="H212" s="7" t="n">
-        <v>46096.71458333333</v>
-      </c>
-      <c r="I212" s="7" t="n"/>
+        <v>45454.79166666666</v>
+      </c>
+      <c r="I212" s="7" t="n">
+        <v>45454.79166666666</v>
+      </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>WAPSA</t>
+          <t>Wapsa Web</t>
         </is>
       </c>
       <c r="K212" t="inlineStr"/>
       <c r="L212" t="n">
-        <v>485</v>
+        <v>358</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>Frank Macavilca &lt;dmacavilca@syc-sistemas.com&gt;</t>
+          <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>&lt;div&gt;&lt;b&gt;Descripción:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;He registrado el ultimo movimiento de esa ruma a las 23:00 hrs del 14/03, el ajuste lo estoy poniendo como 14/03 23:59, por que si le pongo 15/03 que fue en realidad la operación me sale otro error que dice que la fecha no puede ser posterior a la fecha de resumen&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/9970cbf3-cd07-41b8-8c16-d3ff09d6b2f6?fileName=image.png" alt=Image&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;Solución:&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;&lt;div&gt;&lt;b&gt;&lt;br&gt;&lt;/b&gt; &lt;/div&gt;</t>
+          <t>&lt;div&gt;Nicolas solicitar completar infromacion resulotante de uan reunion con Chnalco sobre propuestas de mejoras acerca de los Pases a produccion, tickets y ambientes de pruebas &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/5ee0bb74-9fda-4771-adab-e78824534323?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Reunion con NV y DM para revisar propuestas de mejoras. &lt;/div&gt;&lt;div&gt;12/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp; Se envian propuestas a evaluacion de NV &lt;/div&gt;</t>
         </is>
       </c>
       <c r="O212" t="inlineStr">
@@ -23874,12 +23898,12 @@
       </c>
       <c r="P212" t="inlineStr">
         <is>
-          <t>S&amp;C Sistemas</t>
+          <t>Externos</t>
         </is>
       </c>
       <c r="Q212" t="inlineStr">
         <is>
-          <t>Estabilización por proyecto</t>
+          <t>No implica estabilización</t>
         </is>
       </c>
       <c r="R212" t="n">
@@ -23893,7 +23917,7 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>255</v>
+        <v>340</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -23902,29 +23926,25 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Ticket 358 - Wapsa - General - Informacion sobre propuesta de mejoras para los Pases a produccion, tickets y ambientes de pruebas</t>
+          <t>Ticket 384 - Wapsa - General - Configuracion -  Crear Modulo para guardar las plantilla de importacion de datos</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>WAPSA\Sprint - Junio 2024</t>
+          <t>WAPSA\Sprint - Junio - 2026</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Cerrado</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" s="7" t="n">
-        <v>45453.79166666666</v>
-      </c>
-      <c r="H213" s="7" t="n">
-        <v>45454.79166666666</v>
-      </c>
-      <c r="I213" s="7" t="n">
-        <v>45454.79166666666</v>
-      </c>
+        <v>45951.79166666666</v>
+      </c>
+      <c r="H213" s="7" t="n"/>
+      <c r="I213" s="7" t="n"/>
       <c r="J213" t="inlineStr">
         <is>
           <t>Wapsa Web</t>
@@ -23932,18 +23952,14 @@
       </c>
       <c r="K213" t="inlineStr"/>
       <c r="L213" t="n">
-        <v>358</v>
+        <v>384</v>
       </c>
       <c r="M213" t="inlineStr">
         <is>
           <t>Cristian Pastor Artigas &lt;cartigas@syc-sistemas.com&gt;</t>
         </is>
       </c>
-      <c r="N213" t="inlineStr">
-        <is>
-          <t>&lt;div&gt;Nicolas solicitar completar infromacion resulotante de uan reunion con Chnalco sobre propuestas de mejoras acerca de los Pases a produccion, tickets y ambientes de pruebas &lt;/div&gt;&lt;div&gt;&lt;img src="https://dev.azure.com/SycSistemas/833274e7-44d5-4093-8f90-9bab7903e605/_apis/wit/attachments/5ee0bb74-9fda-4771-adab-e78824534323?fileName=image.png" alt=Image&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;&lt;br&gt; &lt;/div&gt;&lt;div&gt;11/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp;Reunion con NV y DM para revisar propuestas de mejoras. &lt;/div&gt;&lt;div&gt;12/06 &lt;a href="#" data-vss-mention="version:2.0,d542a3a1-6dfe-6329-8f4f-0c05b9f92ebc"&gt;@Cristian Pastor Artigas&lt;/a&gt;&amp;nbsp; Se envian propuestas a evaluacion de NV &lt;/div&gt;</t>
-        </is>
-      </c>
+      <c r="N213" t="inlineStr"/>
       <c r="O213" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -23951,7 +23967,7 @@
       </c>
       <c r="P213" t="inlineStr">
         <is>
-          <t>Externos</t>
+          <t>S&amp;C Sistemas</t>
         </is>
       </c>
       <c r="Q213" t="inlineStr">

</xml_diff>